<commit_message>
Remove helper column R, restore Description as the original column
Column K stays exactly what it was in the source file - the
Description column - just with standardised (typo-fixed) text instead
of a formula. The Colour formula now reads directly from K instead of
a separate raw-text helper column, which is no longer needed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192FU3Scg9XSr7HEGSJ8k2R
</commit_message>
<xml_diff>
--- a/ReBorn_stock_list_26_FINAL.xlsx
+++ b/ReBorn_stock_list_26_FINAL.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="165" formatCode="&quot;£&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -95,10 +95,6 @@
     </font>
     <font>
       <b val="1"/>
-      <i val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <i val="1"/>
@@ -157,7 +153,7 @@
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,16 +219,15 @@
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="4"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -920,7 +915,6 @@
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customFormat="1" customHeight="1" s="5">
@@ -1009,11 +1003,6 @@
           <t>Margin</t>
         </is>
       </c>
-      <c r="R1" s="31" t="inlineStr">
-        <is>
-          <t>Original Description (raw, unedited - for reference)</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1072,27 +1061,22 @@
       <c r="L2" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="M2" s="32" t="n">
+      <c r="M2" s="31" t="n">
         <v>6.95</v>
       </c>
-      <c r="N2" s="32" t="n">
+      <c r="N2" s="31" t="n">
         <v>39</v>
       </c>
       <c r="O2" s="17" t="n">
         <v>1.2</v>
       </c>
-      <c r="P2" s="33">
+      <c r="P2" s="32">
         <f>SUM(N2/O2)</f>
         <v/>
       </c>
-      <c r="Q2" s="34">
+      <c r="Q2" s="33">
         <f>((N2/O2)-M2)/(N2/O2)</f>
         <v/>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Cashmere Fingerless Gloves Aubergine</t>
-        </is>
       </c>
       <c r="Y2" s="19" t="n"/>
       <c r="Z2" s="19" t="n"/>
@@ -1127,13 +1111,13 @@
         <f>"Cashmere "&amp;E3</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H3" s="35" t="inlineStr">
+      <c r="H3" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I3" t="str">
-        <f>TRIM(MID(R3,FIND(",",R3)+1,FIND(",",R3,FIND(",",R3)+1)-FIND(",",R3)-1))</f>
+        <f>TRIM(MID(K3,FIND(",",K3)+1,FIND(",",K3,FIND(",",K3)+1)-FIND(",",K3)-1))</f>
         <v>Black</v>
       </c>
       <c r="J3" t="inlineStr">
@@ -1141,9 +1125,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K3" t="str">
-        <f>VLOOKUP(B3,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I3&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Black, O/S</v>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Black, O/S</t>
+        </is>
       </c>
       <c r="L3" t="n">
         <v>6600</v>
@@ -1168,11 +1153,6 @@
         <f>IF(AND(ISNUMBER(N3),ISNUMBER(O3),ISNUMBER(M3)),((N3/O3)-M3)/(N3/O3),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Black, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1204,13 +1184,13 @@
         <f>"Cashmere "&amp;E4</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H4" s="35" t="inlineStr">
+      <c r="H4" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I4" t="str">
-        <f>TRIM(MID(R4,FIND(",",R4)+1,FIND(",",R4,FIND(",",R4)+1)-FIND(",",R4)-1))</f>
+        <f>TRIM(MID(K4,FIND(",",K4)+1,FIND(",",K4,FIND(",",K4)+1)-FIND(",",K4)-1))</f>
         <v>Light Grey</v>
       </c>
       <c r="J4" t="inlineStr">
@@ -1218,9 +1198,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K4" t="str">
-        <f>VLOOKUP(B4,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I4&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Light Grey, O/S</v>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Light Grey, O/S</t>
+        </is>
       </c>
       <c r="L4" t="n">
         <v>3605</v>
@@ -1245,11 +1226,6 @@
         <f>IF(AND(ISNUMBER(N4),ISNUMBER(O4),ISNUMBER(M4)),((N4/O4)-M4)/(N4/O4),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Light Grey, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1281,13 +1257,13 @@
         <f>"Cashmere "&amp;E5</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H5" s="35" t="inlineStr">
+      <c r="H5" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I5" t="str">
-        <f>TRIM(MID(R5,FIND(",",R5)+1,FIND(",",R5,FIND(",",R5)+1)-FIND(",",R5)-1))</f>
+        <f>TRIM(MID(K5,FIND(",",K5)+1,FIND(",",K5,FIND(",",K5)+1)-FIND(",",K5)-1))</f>
         <v>Dark Grey</v>
       </c>
       <c r="J5" t="inlineStr">
@@ -1295,9 +1271,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K5" t="str">
-        <f>VLOOKUP(B5,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I5&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Dark Grey, O/S</v>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Dark Grey, O/S</t>
+        </is>
       </c>
       <c r="L5" t="n">
         <v>3599</v>
@@ -1322,11 +1299,6 @@
         <f>IF(AND(ISNUMBER(N5),ISNUMBER(O5),ISNUMBER(M5)),((N5/O5)-M5)/(N5/O5),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Dark Grey, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1358,13 +1330,13 @@
         <f>"Cashmere "&amp;E6</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H6" s="35" t="inlineStr">
+      <c r="H6" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I6" t="str">
-        <f>TRIM(MID(R6,FIND(",",R6)+1,FIND(",",R6,FIND(",",R6)+1)-FIND(",",R6)-1))</f>
+        <f>TRIM(MID(K6,FIND(",",K6)+1,FIND(",",K6,FIND(",",K6)+1)-FIND(",",K6)-1))</f>
         <v>Light Beige</v>
       </c>
       <c r="J6" t="inlineStr">
@@ -1372,9 +1344,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K6" t="str">
-        <f>VLOOKUP(B6,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I6&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Light Beige, O/S</v>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Light Beige, O/S</t>
+        </is>
       </c>
       <c r="L6" t="n">
         <v>3018</v>
@@ -1399,11 +1372,6 @@
         <f>IF(AND(ISNUMBER(N6),ISNUMBER(O6),ISNUMBER(M6)),((N6/O6)-M6)/(N6/O6),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Light Beige, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1435,13 +1403,13 @@
         <f>"Cashmere "&amp;E7</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H7" s="35" t="inlineStr">
+      <c r="H7" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I7" t="str">
-        <f>TRIM(MID(R7,FIND(",",R7)+1,FIND(",",R7,FIND(",",R7)+1)-FIND(",",R7)-1))</f>
+        <f>TRIM(MID(K7,FIND(",",K7)+1,FIND(",",K7,FIND(",",K7)+1)-FIND(",",K7)-1))</f>
         <v>Light Brown</v>
       </c>
       <c r="J7" t="inlineStr">
@@ -1449,9 +1417,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K7" s="27" t="str">
-        <f>VLOOKUP(B7,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I7&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Light Brown, O/S</v>
+      <c r="K7" s="27" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Light Brown, O/S</t>
+        </is>
       </c>
       <c r="L7" t="n">
         <v>1302</v>
@@ -1476,11 +1445,6 @@
         <f>IF(AND(ISNUMBER(N7),ISNUMBER(O7),ISNUMBER(M7)),((N7/O7)-M7)/(N7/O7),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Light Brown, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1512,13 +1476,13 @@
         <f>"Cashmere "&amp;E8</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H8" s="36" t="inlineStr">
+      <c r="H8" s="35" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I8" s="1" t="str">
-        <f>TRIM(MID(R8,FIND(",",R8)+1,FIND(",",R8,FIND(",",R8)+1)-FIND(",",R8)-1))</f>
+        <f>TRIM(MID(K8,FIND(",",K8)+1,FIND(",",K8,FIND(",",K8)+1)-FIND(",",K8)-1))</f>
         <v>Navy</v>
       </c>
       <c r="J8" s="1" t="inlineStr">
@@ -1526,9 +1490,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K8" t="str">
-        <f>VLOOKUP(B8,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I8&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Navy, O/S</v>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Navy, O/S</t>
+        </is>
       </c>
       <c r="L8" t="n">
         <v>1036</v>
@@ -1553,11 +1518,7 @@
         <f>IF(AND(ISNUMBER(N8),ISNUMBER(O8),ISNUMBER(M8)),((N8/O8)-M8)/(N8/O8),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R8" s="1" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Navy, O/S</t>
-        </is>
-      </c>
+      <c r="R8" s="1" t="n"/>
       <c r="S8" s="1" t="n"/>
       <c r="T8" s="1" t="n"/>
       <c r="U8" s="1" t="n"/>
@@ -1628,13 +1589,13 @@
         <f>"Cashmere "&amp;E9</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H9" s="35" t="inlineStr">
+      <c r="H9" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I9" t="str">
-        <f>TRIM(MID(R9,FIND(",",R9)+1,FIND(",",R9,FIND(",",R9)+1)-FIND(",",R9)-1))</f>
+        <f>TRIM(MID(K9,FIND(",",K9)+1,FIND(",",K9,FIND(",",K9)+1)-FIND(",",K9)-1))</f>
         <v>Light Maroon</v>
       </c>
       <c r="J9" t="inlineStr">
@@ -1642,9 +1603,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K9" t="str">
-        <f>VLOOKUP(B9,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I9&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Light Maroon, O/S</v>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Light Maroon, O/S</t>
+        </is>
       </c>
       <c r="L9" t="n">
         <v>991</v>
@@ -1669,11 +1631,6 @@
         <f>IF(AND(ISNUMBER(N9),ISNUMBER(O9),ISNUMBER(M9)),((N9/O9)-M9)/(N9/O9),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Light Maroon, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1705,13 +1662,13 @@
         <f>"Cashmere "&amp;E10</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H10" s="36" t="inlineStr">
+      <c r="H10" s="35" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I10" s="1" t="str">
-        <f>TRIM(MID(R10,FIND(",",R10)+1,FIND(",",R10,FIND(",",R10)+1)-FIND(",",R10)-1))</f>
+        <f>TRIM(MID(K10,FIND(",",K10)+1,FIND(",",K10,FIND(",",K10)+1)-FIND(",",K10)-1))</f>
         <v>Red</v>
       </c>
       <c r="J10" s="1" t="inlineStr">
@@ -1719,9 +1676,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K10" t="str">
-        <f>VLOOKUP(B10,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I10&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Red, O/S</v>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Red, O/S</t>
+        </is>
       </c>
       <c r="L10" t="n">
         <v>988</v>
@@ -1746,11 +1704,7 @@
         <f>IF(AND(ISNUMBER(N10),ISNUMBER(O10),ISNUMBER(M10)),((N10/O10)-M10)/(N10/O10),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R10" s="1" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Red, O/S</t>
-        </is>
-      </c>
+      <c r="R10" s="1" t="n"/>
       <c r="S10" s="1" t="n"/>
       <c r="T10" s="1" t="n"/>
       <c r="U10" s="1" t="n"/>
@@ -1821,13 +1775,13 @@
         <f>"Cashmere "&amp;E11</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H11" s="35" t="inlineStr">
+      <c r="H11" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I11" t="str">
-        <f>TRIM(MID(R11,FIND(",",R11)+1,FIND(",",R11,FIND(",",R11)+1)-FIND(",",R11)-1))</f>
+        <f>TRIM(MID(K11,FIND(",",K11)+1,FIND(",",K11,FIND(",",K11)+1)-FIND(",",K11)-1))</f>
         <v>Baby Pink</v>
       </c>
       <c r="J11" t="inlineStr">
@@ -1835,9 +1789,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K11" t="str">
-        <f>VLOOKUP(B11,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I11&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Baby Pink, O/S</v>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Baby Pink, O/S</t>
+        </is>
       </c>
       <c r="L11" t="n">
         <v>800</v>
@@ -1862,11 +1817,6 @@
         <f>IF(AND(ISNUMBER(N11),ISNUMBER(O11),ISNUMBER(M11)),((N11/O11)-M11)/(N11/O11),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Baby Pink, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1898,13 +1848,13 @@
         <f>"Cashmere "&amp;E12</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H12" s="35" t="inlineStr">
+      <c r="H12" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I12" t="str">
-        <f>TRIM(MID(R12,FIND(",",R12)+1,FIND(",",R12,FIND(",",R12)+1)-FIND(",",R12)-1))</f>
+        <f>TRIM(MID(K12,FIND(",",K12)+1,FIND(",",K12,FIND(",",K12)+1)-FIND(",",K12)-1))</f>
         <v>Dark Brown</v>
       </c>
       <c r="J12" t="inlineStr">
@@ -1912,9 +1862,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K12" t="str">
-        <f>VLOOKUP(B12,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I12&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Dark Brown, O/S</v>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Dark Brown, O/S</t>
+        </is>
       </c>
       <c r="L12" t="n">
         <v>740</v>
@@ -1939,11 +1890,6 @@
         <f>IF(AND(ISNUMBER(N12),ISNUMBER(O12),ISNUMBER(M12)),((N12/O12)-M12)/(N12/O12),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Dark Brown, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1975,13 +1921,13 @@
         <f>"Cashmere "&amp;E13</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H13" s="35" t="inlineStr">
+      <c r="H13" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I13" t="str">
-        <f>TRIM(MID(R13,FIND(",",R13)+1,FIND(",",R13,FIND(",",R13)+1)-FIND(",",R13)-1))</f>
+        <f>TRIM(MID(K13,FIND(",",K13)+1,FIND(",",K13,FIND(",",K13)+1)-FIND(",",K13)-1))</f>
         <v>Yellow</v>
       </c>
       <c r="J13" t="inlineStr">
@@ -1989,9 +1935,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K13" t="str">
-        <f>VLOOKUP(B13,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I13&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Yellow, O/S</v>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Yellow, O/S</t>
+        </is>
       </c>
       <c r="L13" t="n">
         <v>736</v>
@@ -2016,11 +1963,6 @@
         <f>IF(AND(ISNUMBER(N13),ISNUMBER(O13),ISNUMBER(M13)),((N13/O13)-M13)/(N13/O13),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Yellow, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2052,13 +1994,13 @@
         <f>"Cashmere "&amp;E14</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H14" s="35" t="inlineStr">
+      <c r="H14" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I14" t="str">
-        <f>TRIM(MID(R14,FIND(",",R14)+1,FIND(",",R14,FIND(",",R14)+1)-FIND(",",R14)-1))</f>
+        <f>TRIM(MID(K14,FIND(",",K14)+1,FIND(",",K14,FIND(",",K14)+1)-FIND(",",K14)-1))</f>
         <v>Beige</v>
       </c>
       <c r="J14" t="inlineStr">
@@ -2066,9 +2008,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K14" t="str">
-        <f>VLOOKUP(B14,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I14&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Beige, O/S</v>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Beige, O/S</t>
+        </is>
       </c>
       <c r="L14" t="n">
         <v>624</v>
@@ -2093,11 +2036,6 @@
         <f>IF(AND(ISNUMBER(N14),ISNUMBER(O14),ISNUMBER(M14)),((N14/O14)-M14)/(N14/O14),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Beige, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2129,13 +2067,13 @@
         <f>"Cashmere "&amp;E15</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H15" s="35" t="inlineStr">
+      <c r="H15" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I15" t="str">
-        <f>TRIM(MID(R15,FIND(",",R15)+1,FIND(",",R15,FIND(",",R15)+1)-FIND(",",R15)-1))</f>
+        <f>TRIM(MID(K15,FIND(",",K15)+1,FIND(",",K15,FIND(",",K15)+1)-FIND(",",K15)-1))</f>
         <v>Deep Matcha Green</v>
       </c>
       <c r="J15" t="inlineStr">
@@ -2143,9 +2081,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K15" t="str">
-        <f>VLOOKUP(B15,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I15&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Deep Matcha Green, O/S</v>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Deep Matcha Green, O/S</t>
+        </is>
       </c>
       <c r="L15" t="n">
         <v>598</v>
@@ -2170,11 +2109,6 @@
         <f>IF(AND(ISNUMBER(N15),ISNUMBER(O15),ISNUMBER(M15)),((N15/O15)-M15)/(N15/O15),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Deep Matcha Green, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2206,13 +2140,13 @@
         <f>"Cashmere "&amp;E16</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H16" s="35" t="inlineStr">
+      <c r="H16" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I16" t="str">
-        <f>TRIM(MID(R16,FIND(",",R16)+1,FIND(",",R16,FIND(",",R16)+1)-FIND(",",R16)-1))</f>
+        <f>TRIM(MID(K16,FIND(",",K16)+1,FIND(",",K16,FIND(",",K16)+1)-FIND(",",K16)-1))</f>
         <v>Pink</v>
       </c>
       <c r="J16" t="inlineStr">
@@ -2220,9 +2154,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K16" s="26" t="str">
-        <f>VLOOKUP(B16,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I16&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Pink, O/S</v>
+      <c r="K16" s="26" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Pink, O/S</t>
+        </is>
       </c>
       <c r="L16" t="n">
         <v>534</v>
@@ -2247,11 +2182,6 @@
         <f>IF(AND(ISNUMBER(N16),ISNUMBER(O16),ISNUMBER(M16)),((N16/O16)-M16)/(N16/O16),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Pink, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2283,13 +2213,13 @@
         <f>"Cashmere "&amp;E17</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H17" s="35" t="inlineStr">
+      <c r="H17" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I17" t="str">
-        <f>TRIM(MID(R17,FIND(",",R17)+1,FIND(",",R17,FIND(",",R17)+1)-FIND(",",R17)-1))</f>
+        <f>TRIM(MID(K17,FIND(",",K17)+1,FIND(",",K17,FIND(",",K17)+1)-FIND(",",K17)-1))</f>
         <v>Military Green</v>
       </c>
       <c r="J17" t="inlineStr">
@@ -2297,9 +2227,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K17" s="26" t="str">
-        <f>VLOOKUP(B17,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I17&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Military Green, O/S</v>
+      <c r="K17" s="26" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Military Green, O/S</t>
+        </is>
       </c>
       <c r="L17" t="n">
         <v>525</v>
@@ -2324,11 +2255,6 @@
         <f>IF(AND(ISNUMBER(N17),ISNUMBER(O17),ISNUMBER(M17)),((N17/O17)-M17)/(N17/O17),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Military Green, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2360,13 +2286,13 @@
         <f>"Cashmere "&amp;E18</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H18" s="35" t="inlineStr">
+      <c r="H18" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I18" t="str">
-        <f>TRIM(MID(R18,FIND(",",R18)+1,FIND(",",R18,FIND(",",R18)+1)-FIND(",",R18)-1))</f>
+        <f>TRIM(MID(K18,FIND(",",K18)+1,FIND(",",K18,FIND(",",K18)+1)-FIND(",",K18)-1))</f>
         <v>Light Green</v>
       </c>
       <c r="J18" t="inlineStr">
@@ -2374,9 +2300,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K18" s="26" t="str">
-        <f>VLOOKUP(B18,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I18&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Light Green, O/S</v>
+      <c r="K18" s="26" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Light Green, O/S</t>
+        </is>
       </c>
       <c r="L18" t="n">
         <v>445</v>
@@ -2401,11 +2328,6 @@
         <f>IF(AND(ISNUMBER(N18),ISNUMBER(O18),ISNUMBER(M18)),((N18/O18)-M18)/(N18/O18),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Light Green, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2437,13 +2359,13 @@
         <f>"Cashmere "&amp;E19</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H19" s="35" t="inlineStr">
+      <c r="H19" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I19" t="str">
-        <f>TRIM(MID(R19,FIND(",",R19)+1,FIND(",",R19,FIND(",",R19)+1)-FIND(",",R19)-1))</f>
+        <f>TRIM(MID(K19,FIND(",",K19)+1,FIND(",",K19,FIND(",",K19)+1)-FIND(",",K19)-1))</f>
         <v>Light Blue</v>
       </c>
       <c r="J19" t="inlineStr">
@@ -2451,9 +2373,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K19" s="26" t="str">
-        <f>VLOOKUP(B19,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I19&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Light Blue, O/S</v>
+      <c r="K19" s="26" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Light Blue, O/S</t>
+        </is>
       </c>
       <c r="L19" t="n">
         <v>418</v>
@@ -2478,11 +2401,6 @@
         <f>IF(AND(ISNUMBER(N19),ISNUMBER(O19),ISNUMBER(M19)),((N19/O19)-M19)/(N19/O19),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Light Blue, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2514,13 +2432,13 @@
         <f>"Cashmere "&amp;E20</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H20" s="35" t="inlineStr">
+      <c r="H20" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I20" t="str">
-        <f>TRIM(MID(R20,FIND(",",R20)+1,FIND(",",R20,FIND(",",R20)+1)-FIND(",",R20)-1))</f>
+        <f>TRIM(MID(K20,FIND(",",K20)+1,FIND(",",K20,FIND(",",K20)+1)-FIND(",",K20)-1))</f>
         <v>Lavender</v>
       </c>
       <c r="J20" t="inlineStr">
@@ -2528,9 +2446,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K20" s="26" t="str">
-        <f>VLOOKUP(B20,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I20&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Lavender, O/S</v>
+      <c r="K20" s="26" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Lavender, O/S</t>
+        </is>
       </c>
       <c r="L20" t="n">
         <v>377</v>
@@ -2555,11 +2474,6 @@
         <f>IF(AND(ISNUMBER(N20),ISNUMBER(O20),ISNUMBER(M20)),((N20/O20)-M20)/(N20/O20),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Lavender, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="28" t="inlineStr">
@@ -2591,13 +2505,13 @@
         <f>"Cashmere "&amp;E21</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H21" s="35" t="inlineStr">
+      <c r="H21" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I21" t="str">
-        <f>TRIM(MID(R21,FIND(",",R21)+1,FIND(",",R21,FIND(",",R21)+1)-FIND(",",R21)-1))</f>
+        <f>TRIM(MID(K21,FIND(",",K21)+1,FIND(",",K21,FIND(",",K21)+1)-FIND(",",K21)-1))</f>
         <v>Maroon</v>
       </c>
       <c r="J21" t="inlineStr">
@@ -2605,9 +2519,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K21" t="str">
-        <f>VLOOKUP(B21,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I21&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Maroon, O/S</v>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Maroon, O/S</t>
+        </is>
       </c>
       <c r="L21" t="n">
         <v>365</v>
@@ -2632,11 +2547,6 @@
         <f>IF(AND(ISNUMBER(N21),ISNUMBER(O21),ISNUMBER(M21)),((N21/O21)-M21)/(N21/O21),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Maroon, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2668,13 +2578,13 @@
         <f>"Cashmere "&amp;E22</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H22" s="35" t="inlineStr">
+      <c r="H22" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I22" t="str">
-        <f>TRIM(MID(R22,FIND(",",R22)+1,FIND(",",R22,FIND(",",R22)+1)-FIND(",",R22)-1))</f>
+        <f>TRIM(MID(K22,FIND(",",K22)+1,FIND(",",K22,FIND(",",K22)+1)-FIND(",",K22)-1))</f>
         <v>Denim Blue</v>
       </c>
       <c r="J22" t="inlineStr">
@@ -2682,9 +2592,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K22" t="str">
-        <f>VLOOKUP(B22,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I22&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Denim Blue, O/S</v>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Denim Blue, O/S</t>
+        </is>
       </c>
       <c r="L22" t="n">
         <v>355</v>
@@ -2709,11 +2620,6 @@
         <f>IF(AND(ISNUMBER(N22),ISNUMBER(O22),ISNUMBER(M22)),((N22/O22)-M22)/(N22/O22),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Denim Blue, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2745,13 +2651,13 @@
         <f>"Cashmere "&amp;E23</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H23" s="35" t="inlineStr">
+      <c r="H23" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I23" t="str">
-        <f>TRIM(MID(R23,FIND(",",R23)+1,FIND(",",R23,FIND(",",R23)+1)-FIND(",",R23)-1))</f>
+        <f>TRIM(MID(K23,FIND(",",K23)+1,FIND(",",K23,FIND(",",K23)+1)-FIND(",",K23)-1))</f>
         <v>Kelly Green</v>
       </c>
       <c r="J23" t="inlineStr">
@@ -2759,9 +2665,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K23" t="str">
-        <f>VLOOKUP(B23,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I23&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Kelly Green, O/S</v>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Kelly Green, O/S</t>
+        </is>
       </c>
       <c r="L23" t="n">
         <v>121</v>
@@ -2786,11 +2693,6 @@
         <f>IF(AND(ISNUMBER(N23),ISNUMBER(O23),ISNUMBER(M23)),((N23/O23)-M23)/(N23/O23),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Kelly Green, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2822,13 +2724,13 @@
         <f>"Cashmere "&amp;E24</f>
         <v>Cashmere Beanie &amp; Glove Set</v>
       </c>
-      <c r="H24" s="35" t="inlineStr">
+      <c r="H24" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I24" t="str">
-        <f>TRIM(MID(R24,FIND(",",R24)+1,FIND(",",R24,FIND(",",R24)+1)-FIND(",",R24)-1))</f>
+        <f>TRIM(MID(K24,FIND(",",K24)+1,FIND(",",K24,FIND(",",K24)+1)-FIND(",",K24)-1))</f>
         <v>Black &amp; Red</v>
       </c>
       <c r="J24" t="inlineStr">
@@ -2836,9 +2738,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K24" t="str">
-        <f>VLOOKUP(B24,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I24&amp;", O/S"</f>
-        <v>Re:Born Beanie &amp; Glove Set, Black &amp; Red, O/S</v>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Re:Born Beanie &amp; Glove Set, Black &amp; Red, O/S</t>
+        </is>
       </c>
       <c r="L24" t="n">
         <v>117</v>
@@ -2863,11 +2766,6 @@
         <f>IF(AND(ISNUMBER(N24),ISNUMBER(O24),ISNUMBER(M24)),((N24/O24)-M24)/(N24/O24),"TBC")</f>
         <v>TBC</v>
       </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>Re:Born Beanie &amp; Glove Set, Black &amp; Red, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2899,13 +2797,13 @@
         <f>"Cashmere "&amp;E25</f>
         <v>Cashmere 2 Pack Gloves</v>
       </c>
-      <c r="H25" s="35" t="inlineStr">
+      <c r="H25" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I25" t="str">
-        <f>TRIM(MID(R25,FIND(",",R25)+1,FIND(",",R25,FIND(",",R25)+1)-FIND(",",R25)-1))</f>
+        <f>TRIM(MID(K25,FIND(",",K25)+1,FIND(",",K25,FIND(",",K25)+1)-FIND(",",K25)-1))</f>
         <v>Red And Navy</v>
       </c>
       <c r="J25" t="inlineStr">
@@ -2913,9 +2811,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K25" t="str">
-        <f>VLOOKUP(B25,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I25&amp;", O/S"</f>
-        <v>Re:Born 2 Pack Gloves, Red And Navy, O/S</v>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Re:Born 2 Pack Gloves, Red And Navy, O/S</t>
+        </is>
       </c>
       <c r="L25" t="n">
         <v>98</v>
@@ -2940,11 +2839,6 @@
         <f>IF(AND(ISNUMBER(N25),ISNUMBER(O25),ISNUMBER(M25)),((N25/O25)-M25)/(N25/O25),"TBC")</f>
         <v>TBC</v>
       </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Re:Born 2 Pack Gloves, Red And Navy, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2976,13 +2870,13 @@
         <f>"Cashmere "&amp;E26</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H26" s="35" t="inlineStr">
+      <c r="H26" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I26" t="str">
-        <f>TRIM(MID(R26,FIND(",",R26)+1,FIND(",",R26,FIND(",",R26)+1)-FIND(",",R26)-1))</f>
+        <f>TRIM(MID(K26,FIND(",",K26)+1,FIND(",",K26,FIND(",",K26)+1)-FIND(",",K26)-1))</f>
         <v>Hot Pink</v>
       </c>
       <c r="J26" t="inlineStr">
@@ -2990,9 +2884,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K26" t="str">
-        <f>VLOOKUP(B26,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I26&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Hot Pink, O/S</v>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Hot Pink, O/S</t>
+        </is>
       </c>
       <c r="L26" t="n">
         <v>81</v>
@@ -3017,11 +2912,6 @@
         <f>IF(AND(ISNUMBER(N26),ISNUMBER(O26),ISNUMBER(M26)),((N26/O26)-M26)/(N26/O26),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Hot Pink, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3053,13 +2943,13 @@
         <f>"Cashmere "&amp;E27</f>
         <v>Cashmere 2 Pack Gloves</v>
       </c>
-      <c r="H27" s="35" t="inlineStr">
+      <c r="H27" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I27" t="str">
-        <f>TRIM(MID(R27,FIND(",",R27)+1,FIND(",",R27,FIND(",",R27)+1)-FIND(",",R27)-1))</f>
+        <f>TRIM(MID(K27,FIND(",",K27)+1,FIND(",",K27,FIND(",",K27)+1)-FIND(",",K27)-1))</f>
         <v>Black And Caramel</v>
       </c>
       <c r="J27" t="inlineStr">
@@ -3067,9 +2957,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K27" t="str">
-        <f>VLOOKUP(B27,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I27&amp;", O/S"</f>
-        <v>Re:Born 2 Pack Gloves, Black And Caramel, O/S</v>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Re:Born 2 Pack Gloves, Black And Caramel, O/S</t>
+        </is>
       </c>
       <c r="L27" t="n">
         <v>41</v>
@@ -3094,11 +2985,6 @@
         <f>IF(AND(ISNUMBER(N27),ISNUMBER(O27),ISNUMBER(M27)),((N27/O27)-M27)/(N27/O27),"TBC")</f>
         <v>TBC</v>
       </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>Re:Born 2 Pack Gloves, Black And Caramel, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3130,13 +3016,13 @@
         <f>"Cashmere "&amp;E28</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H28" s="35" t="inlineStr">
+      <c r="H28" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I28" t="str">
-        <f>TRIM(MID(R28,FIND(",",R28)+1,FIND(",",R28,FIND(",",R28)+1)-FIND(",",R28)-1))</f>
+        <f>TRIM(MID(K28,FIND(",",K28)+1,FIND(",",K28,FIND(",",K28)+1)-FIND(",",K28)-1))</f>
         <v>One Of A Kind</v>
       </c>
       <c r="J28" t="inlineStr">
@@ -3144,9 +3030,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K28" t="str">
-        <f>VLOOKUP(B28,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I28&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, One Of A Kind, O/S</v>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, One Of A Kind, O/S</t>
+        </is>
       </c>
       <c r="L28" t="n">
         <v>41</v>
@@ -3171,11 +3058,6 @@
         <f>IF(AND(ISNUMBER(N28),ISNUMBER(O28),ISNUMBER(M28)),((N28/O28)-M28)/(N28/O28),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, One Of A Kind, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3207,13 +3089,13 @@
         <f>"Cashmere "&amp;E29</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H29" s="35" t="inlineStr">
+      <c r="H29" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I29" t="str">
-        <f>TRIM(MID(R29,FIND(",",R29)+1,FIND(",",R29,FIND(",",R29)+1)-FIND(",",R29)-1))</f>
+        <f>TRIM(MID(K29,FIND(",",K29)+1,FIND(",",K29,FIND(",",K29)+1)-FIND(",",K29)-1))</f>
         <v>Brights</v>
       </c>
       <c r="J29" t="inlineStr">
@@ -3221,9 +3103,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K29" t="str">
-        <f>VLOOKUP(B29,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I29&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Brights, O/S</v>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Brights, O/S</t>
+        </is>
       </c>
       <c r="L29" t="n">
         <v>33</v>
@@ -3248,11 +3131,6 @@
         <f>IF(AND(ISNUMBER(N29),ISNUMBER(O29),ISNUMBER(M29)),((N29/O29)-M29)/(N29/O29),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Brights, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3284,13 +3162,13 @@
         <f>"Cashmere "&amp;E30</f>
         <v>Cashmere Beanie &amp; Glove Set</v>
       </c>
-      <c r="H30" s="35" t="inlineStr">
+      <c r="H30" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I30" t="str">
-        <f>TRIM(MID(R30,FIND(",",R30)+1,FIND(",",R30,FIND(",",R30)+1)-FIND(",",R30)-1))</f>
+        <f>TRIM(MID(K30,FIND(",",K30)+1,FIND(",",K30,FIND(",",K30)+1)-FIND(",",K30)-1))</f>
         <v>Navy And Beige</v>
       </c>
       <c r="J30" t="inlineStr">
@@ -3298,9 +3176,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K30" t="str">
-        <f>VLOOKUP(B30,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I30&amp;", O/S"</f>
-        <v>Re:Born Beanie &amp; Glove Set, Navy And Beige, O/S</v>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Re:Born Beanie &amp; Glove Set, Navy And Beige, O/S</t>
+        </is>
       </c>
       <c r="L30" t="n">
         <v>30</v>
@@ -3325,11 +3204,6 @@
         <f>IF(AND(ISNUMBER(N30),ISNUMBER(O30),ISNUMBER(M30)),((N30/O30)-M30)/(N30/O30),"TBC")</f>
         <v>TBC</v>
       </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>Re:Born Beanie &amp; Glove Set, Navy And Beige, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3361,13 +3235,13 @@
         <f>"Cashmere "&amp;E31</f>
         <v>Cashmere Reversible Beanie</v>
       </c>
-      <c r="H31" s="35" t="inlineStr">
+      <c r="H31" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I31" t="str">
-        <f>TRIM(MID(R31,FIND(",",R31)+1,FIND(",",R31,FIND(",",R31)+1)-FIND(",",R31)-1))</f>
+        <f>TRIM(MID(K31,FIND(",",K31)+1,FIND(",",K31,FIND(",",K31)+1)-FIND(",",K31)-1))</f>
         <v>Light Blue&amp;Light Beige</v>
       </c>
       <c r="J31" t="inlineStr">
@@ -3375,9 +3249,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K31" t="str">
-        <f>VLOOKUP(B31,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I31&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Beanie, Light Blue&amp;Light Beige, O/S</v>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Beanie, Light Blue&amp;Light Beige, O/S</t>
+        </is>
       </c>
       <c r="L31" t="n">
         <v>13</v>
@@ -3402,11 +3277,6 @@
         <f>IF(AND(ISNUMBER(N31),ISNUMBER(O31),ISNUMBER(M31)),((N31/O31)-M31)/(N31/O31),"TBC")</f>
         <v>0.72</v>
       </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>Re:Born Reverse Cashmere Beanie, Light Blue&amp;Light Beige, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3438,13 +3308,13 @@
         <f>"Cashmere "&amp;E32</f>
         <v>Cashmere Reversible Beanie</v>
       </c>
-      <c r="H32" s="35" t="inlineStr">
+      <c r="H32" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I32" t="str">
-        <f>TRIM(MID(R32,FIND(",",R32)+1,FIND(",",R32,FIND(",",R32)+1)-FIND(",",R32)-1))</f>
+        <f>TRIM(MID(K32,FIND(",",K32)+1,FIND(",",K32,FIND(",",K32)+1)-FIND(",",K32)-1))</f>
         <v>Black And Light Grey</v>
       </c>
       <c r="J32" t="inlineStr">
@@ -3452,9 +3322,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K32" t="str">
-        <f>VLOOKUP(B32,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I32&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Beanie, Black And Light Grey, O/S</v>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Beanie, Black And Light Grey, O/S</t>
+        </is>
       </c>
       <c r="L32" t="n">
         <v>11</v>
@@ -3479,11 +3350,6 @@
         <f>IF(AND(ISNUMBER(N32),ISNUMBER(O32),ISNUMBER(M32)),((N32/O32)-M32)/(N32/O32),"TBC")</f>
         <v>0.72</v>
       </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>Re:Born Reverse Cashmere Beanie, Black And Light Grey, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3515,13 +3381,13 @@
         <f>"Cashmere "&amp;E33</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H33" s="35" t="inlineStr">
+      <c r="H33" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I33" t="str">
-        <f>TRIM(MID(R33,FIND(",",R33)+1,FIND(",",R33,FIND(",",R33)+1)-FIND(",",R33)-1))</f>
+        <f>TRIM(MID(K33,FIND(",",K33)+1,FIND(",",K33,FIND(",",K33)+1)-FIND(",",K33)-1))</f>
         <v>Orange</v>
       </c>
       <c r="J33" t="inlineStr">
@@ -3529,9 +3395,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K33" t="str">
-        <f>VLOOKUP(B33,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I33&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Orange, O/S</v>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Orange, O/S</t>
+        </is>
       </c>
       <c r="L33" t="n">
         <v>7</v>
@@ -3556,11 +3423,6 @@
         <f>IF(AND(ISNUMBER(N33),ISNUMBER(O33),ISNUMBER(M33)),((N33/O33)-M33)/(N33/O33),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Orange, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3592,13 +3454,13 @@
         <f>"Cashmere "&amp;E34</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H34" s="36" t="inlineStr">
+      <c r="H34" s="35" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I34" s="1" t="str">
-        <f>TRIM(MID(R34,FIND(",",R34)+1,FIND(",",R34,FIND(",",R34)+1)-FIND(",",R34)-1))</f>
+        <f>TRIM(MID(K34,FIND(",",K34)+1,FIND(",",K34,FIND(",",K34)+1)-FIND(",",K34)-1))</f>
         <v>Royal Blue</v>
       </c>
       <c r="J34" s="1" t="inlineStr">
@@ -3606,9 +3468,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K34" t="str">
-        <f>VLOOKUP(B34,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I34&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Royal Blue, O/S</v>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Royal Blue, O/S</t>
+        </is>
       </c>
       <c r="L34" t="n">
         <v>7</v>
@@ -3633,11 +3496,7 @@
         <f>IF(AND(ISNUMBER(N34),ISNUMBER(O34),ISNUMBER(M34)),((N34/O34)-M34)/(N34/O34),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R34" s="1" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Royal Blue, O/S</t>
-        </is>
-      </c>
+      <c r="R34" s="1" t="n"/>
       <c r="S34" s="1" t="n"/>
       <c r="T34" s="1" t="n"/>
       <c r="U34" s="1" t="n"/>
@@ -3708,13 +3567,13 @@
         <f>"Cashmere "&amp;E35</f>
         <v>Cashmere Reversible Snood</v>
       </c>
-      <c r="H35" s="35" t="inlineStr">
+      <c r="H35" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I35" t="str">
-        <f>TRIM(MID(R35,FIND(",",R35)+1,FIND(",",R35,FIND(",",R35)+1)-FIND(",",R35)-1))</f>
+        <f>TRIM(MID(K35,FIND(",",K35)+1,FIND(",",K35,FIND(",",K35)+1)-FIND(",",K35)-1))</f>
         <v>Light Beige&amp;Choco Brown</v>
       </c>
       <c r="J35" t="inlineStr">
@@ -3722,9 +3581,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K35" t="str">
-        <f>VLOOKUP(B35,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I35&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Snood, Light Beige&amp;Choco Brown, O/S</v>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Snood, Light Beige&amp;Choco Brown, O/S</t>
+        </is>
       </c>
       <c r="L35" t="n">
         <v>55</v>
@@ -3749,11 +3609,6 @@
         <f>IF(AND(ISNUMBER(N35),ISNUMBER(O35),ISNUMBER(M35)),((N35/O35)-M35)/(N35/O35),"TBC")</f>
         <v>0.74</v>
       </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>Re:Born Reverse Cashmere Snood, Light Beige&amp;Choco Brown, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3785,13 +3640,13 @@
         <f>"Cashmere "&amp;E36</f>
         <v>Cashmere Reversible Beanie</v>
       </c>
-      <c r="H36" s="35" t="inlineStr">
+      <c r="H36" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I36" t="str">
-        <f>TRIM(MID(R36,FIND(",",R36)+1,FIND(",",R36,FIND(",",R36)+1)-FIND(",",R36)-1))</f>
+        <f>TRIM(MID(K36,FIND(",",K36)+1,FIND(",",K36,FIND(",",K36)+1)-FIND(",",K36)-1))</f>
         <v>Baby Pink And Cream</v>
       </c>
       <c r="J36" t="inlineStr">
@@ -3799,9 +3654,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K36" t="str">
-        <f>VLOOKUP(B36,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I36&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Beanie, Baby Pink And Cream, O/S</v>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Beanie, Baby Pink And Cream, O/S</t>
+        </is>
       </c>
       <c r="L36" t="n">
         <v>49</v>
@@ -3826,11 +3682,6 @@
         <f>IF(AND(ISNUMBER(N36),ISNUMBER(O36),ISNUMBER(M36)),((N36/O36)-M36)/(N36/O36),"TBC")</f>
         <v>0.72</v>
       </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>Re:Born Reversible Cashmere Beanie, Baby Pink And Cream, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3862,13 +3713,13 @@
         <f>"Cashmere "&amp;E37</f>
         <v>Cashmere Reversible Beanie</v>
       </c>
-      <c r="H37" s="35" t="inlineStr">
+      <c r="H37" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I37" t="str">
-        <f>TRIM(MID(R37,FIND(",",R37)+1,FIND(",",R37,FIND(",",R37)+1)-FIND(",",R37)-1))</f>
+        <f>TRIM(MID(K37,FIND(",",K37)+1,FIND(",",K37,FIND(",",K37)+1)-FIND(",",K37)-1))</f>
         <v>Purple And Yellow</v>
       </c>
       <c r="J37" t="inlineStr">
@@ -3876,9 +3727,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K37" t="str">
-        <f>VLOOKUP(B37,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I37&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Beanie, Purple And Yellow, O/S</v>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Beanie, Purple And Yellow, O/S</t>
+        </is>
       </c>
       <c r="L37" t="n">
         <v>7</v>
@@ -3903,11 +3755,6 @@
         <f>IF(AND(ISNUMBER(N37),ISNUMBER(O37),ISNUMBER(M37)),((N37/O37)-M37)/(N37/O37),"TBC")</f>
         <v>0.72</v>
       </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>Re:Born Reversible Cashmere Beanie, Purple And Yellow, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3939,13 +3786,13 @@
         <f>"Cashmere "&amp;E38</f>
         <v>Cashmere Reversible Beanie</v>
       </c>
-      <c r="H38" s="35" t="inlineStr">
+      <c r="H38" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I38" t="str">
-        <f>TRIM(MID(R38,FIND(",",R38)+1,FIND(",",R38,FIND(",",R38)+1)-FIND(",",R38)-1))</f>
+        <f>TRIM(MID(K38,FIND(",",K38)+1,FIND(",",K38,FIND(",",K38)+1)-FIND(",",K38)-1))</f>
         <v>Red And Beige</v>
       </c>
       <c r="J38" t="inlineStr">
@@ -3953,9 +3800,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K38" t="str">
-        <f>VLOOKUP(B38,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I38&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Beanie, Red And Beige, O/S</v>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Beanie, Red And Beige, O/S</t>
+        </is>
       </c>
       <c r="L38" t="n">
         <v>26</v>
@@ -3980,11 +3828,6 @@
         <f>IF(AND(ISNUMBER(N38),ISNUMBER(O38),ISNUMBER(M38)),((N38/O38)-M38)/(N38/O38),"TBC")</f>
         <v>0.72</v>
       </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>Re:Born Reversible Cashmere Beanie, Red And Beige, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4016,13 +3859,13 @@
         <f>"Cashmere "&amp;E39</f>
         <v>Cashmere Reversible Snood</v>
       </c>
-      <c r="H39" s="35" t="inlineStr">
+      <c r="H39" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I39" t="str">
-        <f>TRIM(MID(R39,FIND(",",R39)+1,FIND(",",R39,FIND(",",R39)+1)-FIND(",",R39)-1))</f>
+        <f>TRIM(MID(K39,FIND(",",K39)+1,FIND(",",K39,FIND(",",K39)+1)-FIND(",",K39)-1))</f>
         <v>Beige And Brown</v>
       </c>
       <c r="J39" t="inlineStr">
@@ -4030,9 +3873,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K39" t="str">
-        <f>VLOOKUP(B39,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I39&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Snood, Beige And Brown, O/S</v>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Snood, Beige And Brown, O/S</t>
+        </is>
       </c>
       <c r="L39" t="n">
         <v>10</v>
@@ -4057,11 +3901,6 @@
         <f>IF(AND(ISNUMBER(N39),ISNUMBER(O39),ISNUMBER(M39)),((N39/O39)-M39)/(N39/O39),"TBC")</f>
         <v>0.74</v>
       </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>Re:Born Reversible Cashmere Snood, Beige And Brown, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4093,13 +3932,13 @@
         <f>"Cashmere "&amp;E40</f>
         <v>Cashmere Reversible Snood</v>
       </c>
-      <c r="H40" s="35" t="inlineStr">
+      <c r="H40" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I40" t="str">
-        <f>TRIM(MID(R40,FIND(",",R40)+1,FIND(",",R40,FIND(",",R40)+1)-FIND(",",R40)-1))</f>
+        <f>TRIM(MID(K40,FIND(",",K40)+1,FIND(",",K40,FIND(",",K40)+1)-FIND(",",K40)-1))</f>
         <v>Black And Dark Grey</v>
       </c>
       <c r="J40" t="inlineStr">
@@ -4107,9 +3946,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K40" t="str">
-        <f>VLOOKUP(B40,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I40&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Snood, Black And Dark Grey, O/S</v>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Snood, Black And Dark Grey, O/S</t>
+        </is>
       </c>
       <c r="L40" t="n">
         <v>11</v>
@@ -4134,11 +3974,6 @@
         <f>IF(AND(ISNUMBER(N40),ISNUMBER(O40),ISNUMBER(M40)),((N40/O40)-M40)/(N40/O40),"TBC")</f>
         <v>0.74</v>
       </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>Re:Born Reversible Cashmere Snood, Black And Dark Grey, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4170,13 +4005,13 @@
         <f>"Cashmere "&amp;E41</f>
         <v>Cashmere Reversible Snood</v>
       </c>
-      <c r="H41" s="35" t="inlineStr">
+      <c r="H41" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I41" t="str">
-        <f>TRIM(MID(R41,FIND(",",R41)+1,FIND(",",R41,FIND(",",R41)+1)-FIND(",",R41)-1))</f>
+        <f>TRIM(MID(K41,FIND(",",K41)+1,FIND(",",K41,FIND(",",K41)+1)-FIND(",",K41)-1))</f>
         <v>Black</v>
       </c>
       <c r="J41" t="inlineStr">
@@ -4184,9 +4019,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K41" t="str">
-        <f>VLOOKUP(B41,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I41&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Snood, Black, O/S</v>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Snood, Black, O/S</t>
+        </is>
       </c>
       <c r="L41" t="n">
         <v>128</v>
@@ -4211,11 +4047,6 @@
         <f>IF(AND(ISNUMBER(N41),ISNUMBER(O41),ISNUMBER(M41)),((N41/O41)-M41)/(N41/O41),"TBC")</f>
         <v>0.74</v>
       </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>Re:Born Reversible Cashmere Snood, Black, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4247,13 +4078,13 @@
         <f>"Cashmere "&amp;E42</f>
         <v>Cashmere Reversible Snood</v>
       </c>
-      <c r="H42" s="35" t="inlineStr">
+      <c r="H42" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I42" t="str">
-        <f>TRIM(MID(R42,FIND(",",R42)+1,FIND(",",R42,FIND(",",R42)+1)-FIND(",",R42)-1))</f>
+        <f>TRIM(MID(K42,FIND(",",K42)+1,FIND(",",K42,FIND(",",K42)+1)-FIND(",",K42)-1))</f>
         <v>Light Grey And Black</v>
       </c>
       <c r="J42" t="inlineStr">
@@ -4261,9 +4092,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K42" t="str">
-        <f>VLOOKUP(B42,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I42&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Snood, Light Grey And Black, O/S</v>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Snood, Light Grey And Black, O/S</t>
+        </is>
       </c>
       <c r="L42" t="n">
         <v>138</v>
@@ -4288,11 +4120,6 @@
         <f>IF(AND(ISNUMBER(N42),ISNUMBER(O42),ISNUMBER(M42)),((N42/O42)-M42)/(N42/O42),"TBC")</f>
         <v>0.74</v>
       </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>Re:Born Reversible Cashmere Snood, Light Grey And Black, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4324,13 +4151,13 @@
         <f>"Cashmere "&amp;E43</f>
         <v>Cashmere Reversible Snood</v>
       </c>
-      <c r="H43" s="35" t="inlineStr">
+      <c r="H43" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I43" t="str">
-        <f>TRIM(MID(R43,FIND(",",R43)+1,FIND(",",R43,FIND(",",R43)+1)-FIND(",",R43)-1))</f>
+        <f>TRIM(MID(K43,FIND(",",K43)+1,FIND(",",K43,FIND(",",K43)+1)-FIND(",",K43)-1))</f>
         <v>Maroon And Dark Grey</v>
       </c>
       <c r="J43" t="inlineStr">
@@ -4338,9 +4165,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K43" t="str">
-        <f>VLOOKUP(B43,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I43&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Snood, Maroon And Dark Grey, O/S</v>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Snood, Maroon And Dark Grey, O/S</t>
+        </is>
       </c>
       <c r="L43" t="n">
         <v>10</v>
@@ -4365,11 +4193,6 @@
         <f>IF(AND(ISNUMBER(N43),ISNUMBER(O43),ISNUMBER(M43)),((N43/O43)-M43)/(N43/O43),"TBC")</f>
         <v>0.74</v>
       </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Re:Born Reversible Cashmere Snood, Maroon And Dark Grey, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4401,13 +4224,13 @@
         <f>"Cashmere "&amp;E44</f>
         <v>Cashmere Reversible Snood</v>
       </c>
-      <c r="H44" s="35" t="inlineStr">
+      <c r="H44" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I44" t="str">
-        <f>TRIM(MID(R44,FIND(",",R44)+1,FIND(",",R44,FIND(",",R44)+1)-FIND(",",R44)-1))</f>
+        <f>TRIM(MID(K44,FIND(",",K44)+1,FIND(",",K44,FIND(",",K44)+1)-FIND(",",K44)-1))</f>
         <v>Red And Cream</v>
       </c>
       <c r="J44" t="inlineStr">
@@ -4415,9 +4238,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K44" t="str">
-        <f>VLOOKUP(B44,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I44&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Snood, Red And Cream, O/S</v>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Snood, Red And Cream, O/S</t>
+        </is>
       </c>
       <c r="L44" t="n">
         <v>34</v>
@@ -4442,11 +4266,6 @@
         <f>IF(AND(ISNUMBER(N44),ISNUMBER(O44),ISNUMBER(M44)),((N44/O44)-M44)/(N44/O44),"TBC")</f>
         <v>0.74</v>
       </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>Re:Born Reversible Cashmere Snood, Red And Cream, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4478,13 +4297,13 @@
         <f>"Cashmere "&amp;E45</f>
         <v>Cashmere Snood &amp; Glove Set</v>
       </c>
-      <c r="H45" s="35" t="inlineStr">
+      <c r="H45" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I45" t="str">
-        <f>TRIM(MID(R45,FIND(",",R45)+1,FIND(",",R45,FIND(",",R45)+1)-FIND(",",R45)-1))</f>
+        <f>TRIM(MID(K45,FIND(",",K45)+1,FIND(",",K45,FIND(",",K45)+1)-FIND(",",K45)-1))</f>
         <v>Navy/Red and Grey</v>
       </c>
       <c r="J45" t="inlineStr">
@@ -4492,9 +4311,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K45" t="str">
-        <f>VLOOKUP(B45,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I45&amp;", O/S"</f>
-        <v>Re:Born Snood &amp; Glove Set, Navy/Red and Grey, O/S</v>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Re:Born Snood &amp; Glove Set, Navy/Red and Grey, O/S</t>
+        </is>
       </c>
       <c r="L45" t="n">
         <v>35</v>
@@ -4519,11 +4339,6 @@
         <f>IF(AND(ISNUMBER(N45),ISNUMBER(O45),ISNUMBER(M45)),((N45/O45)-M45)/(N45/O45),"TBC")</f>
         <v>TBC</v>
       </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>Re:Born Snood &amp; Glove Set, Navy/Red and Grey, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4555,13 +4370,13 @@
         <f>"Cashmere "&amp;E46</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H46" s="35" t="inlineStr">
+      <c r="H46" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I46" t="str">
-        <f>TRIM(MID(R46,FIND(",",R46)+1,FIND(",",R46,FIND(",",R46)+1)-FIND(",",R46)-1))</f>
+        <f>TRIM(MID(K46,FIND(",",K46)+1,FIND(",",K46,FIND(",",K46)+1)-FIND(",",K46)-1))</f>
         <v>Grape Purple</v>
       </c>
       <c r="J46" t="inlineStr">
@@ -4569,9 +4384,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K46" t="str">
-        <f>VLOOKUP(B46,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I46&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Grape Purple, O/S</v>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Grape Purple, O/S</t>
+        </is>
       </c>
       <c r="L46" t="n">
         <v>277</v>
@@ -4596,11 +4412,6 @@
         <f>IF(AND(ISNUMBER(N46),ISNUMBER(O46),ISNUMBER(M46)),((N46/O46)-M46)/(N46/O46),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Grape Purple, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4632,13 +4443,13 @@
         <f>"Cashmere "&amp;E47</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H47" s="35" t="inlineStr">
+      <c r="H47" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I47" t="str">
-        <f>TRIM(MID(R47,FIND(",",R47)+1,FIND(",",R47,FIND(",",R47)+1)-FIND(",",R47)-1))</f>
+        <f>TRIM(MID(K47,FIND(",",K47)+1,FIND(",",K47,FIND(",",K47)+1)-FIND(",",K47)-1))</f>
         <v>Dark Purple</v>
       </c>
       <c r="J47" t="inlineStr">
@@ -4646,9 +4457,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K47" t="str">
-        <f>VLOOKUP(B47,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I47&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Dark Purple, O/S</v>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Dark Purple, O/S</t>
+        </is>
       </c>
       <c r="L47" t="n">
         <v>230</v>
@@ -4673,11 +4485,6 @@
         <f>IF(AND(ISNUMBER(N47),ISNUMBER(O47),ISNUMBER(M47)),((N47/O47)-M47)/(N47/O47),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Dark Purple, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="48" customFormat="1" s="1">
       <c r="A48" t="inlineStr">
@@ -4709,13 +4516,13 @@
         <f>"Cashmere "&amp;E48</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H48" s="36" t="inlineStr">
+      <c r="H48" s="35" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I48" s="1" t="str">
-        <f>TRIM(MID(R48,FIND(",",R48)+1,FIND(",",R48,FIND(",",R48)+1)-FIND(",",R48)-1))</f>
+        <f>TRIM(MID(K48,FIND(",",K48)+1,FIND(",",K48,FIND(",",K48)+1)-FIND(",",K48)-1))</f>
         <v>Ocean Green</v>
       </c>
       <c r="J48" s="1" t="inlineStr">
@@ -4723,9 +4530,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K48" t="str">
-        <f>VLOOKUP(B48,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I48&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Ocean Green, O/S</v>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Ocean Green, O/S</t>
+        </is>
       </c>
       <c r="L48" t="n">
         <v>229</v>
@@ -4750,11 +4558,7 @@
         <f>IF(AND(ISNUMBER(N48),ISNUMBER(O48),ISNUMBER(M48)),((N48/O48)-M48)/(N48/O48),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R48" s="1" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Ocean Green, O/S</t>
-        </is>
-      </c>
+      <c r="R48" s="1" t="n"/>
       <c r="S48" s="1" t="n"/>
       <c r="T48" s="1" t="n"/>
       <c r="U48" s="1" t="n"/>
@@ -4825,13 +4629,13 @@
         <f>"Cashmere "&amp;E49</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H49" s="35" t="inlineStr">
+      <c r="H49" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I49" t="str">
-        <f>TRIM(MID(R49,FIND(",",R49)+1,FIND(",",R49,FIND(",",R49)+1)-FIND(",",R49)-1))</f>
+        <f>TRIM(MID(K49,FIND(",",K49)+1,FIND(",",K49,FIND(",",K49)+1)-FIND(",",K49)-1))</f>
         <v>Baby Blue</v>
       </c>
       <c r="J49" t="inlineStr">
@@ -4839,9 +4643,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K49" t="str">
-        <f>VLOOKUP(B49,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I49&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Baby Blue, O/S</v>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Baby Blue, O/S</t>
+        </is>
       </c>
       <c r="L49" t="n">
         <v>161</v>
@@ -4866,11 +4671,6 @@
         <f>IF(AND(ISNUMBER(N49),ISNUMBER(O49),ISNUMBER(M49)),((N49/O49)-M49)/(N49/O49),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Baby Blue, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="50" customFormat="1" s="1">
       <c r="A50" t="inlineStr">
@@ -4902,13 +4702,13 @@
         <f>"Cashmere "&amp;E50</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H50" s="35" t="inlineStr">
+      <c r="H50" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I50" t="str">
-        <f>TRIM(MID(R50,FIND(",",R50)+1,FIND(",",R50,FIND(",",R50)+1)-FIND(",",R50)-1))</f>
+        <f>TRIM(MID(K50,FIND(",",K50)+1,FIND(",",K50,FIND(",",K50)+1)-FIND(",",K50)-1))</f>
         <v>Teal</v>
       </c>
       <c r="J50" t="inlineStr">
@@ -4916,9 +4716,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K50" t="str">
-        <f>VLOOKUP(B50,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I50&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Teal, O/S</v>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Teal, O/S</t>
+        </is>
       </c>
       <c r="L50" t="n">
         <v>138</v>
@@ -4943,11 +4744,6 @@
         <f>IF(AND(ISNUMBER(N50),ISNUMBER(O50),ISNUMBER(M50)),((N50/O50)-M50)/(N50/O50),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R50" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Teal, O/S</t>
-        </is>
-      </c>
     </row>
     <row r="51" customFormat="1" s="1">
       <c r="A51" t="inlineStr">
@@ -4979,13 +4775,13 @@
         <f>"Cashmere "&amp;E51</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H51" s="36" t="inlineStr">
+      <c r="H51" s="35" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I51" s="1" t="str">
-        <f>TRIM(MID(R51,FIND(",",R51)+1,FIND(",",R51,FIND(",",R51)+1)-FIND(",",R51)-1))</f>
+        <f>TRIM(MID(K51,FIND(",",K51)+1,FIND(",",K51,FIND(",",K51)+1)-FIND(",",K51)-1))</f>
         <v>Stripes</v>
       </c>
       <c r="J51" s="1" t="inlineStr">
@@ -4993,9 +4789,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K51" t="str">
-        <f>VLOOKUP(B51,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I51&amp;", O/S"</f>
-        <v>Re:Born Cashmere Fingerless Gloves, Stripes, O/S</v>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Re:Born Cashmere Fingerless Gloves, Stripes, O/S</t>
+        </is>
       </c>
       <c r="L51" t="n">
         <v>137</v>
@@ -5020,11 +4817,7 @@
         <f>IF(AND(ISNUMBER(N51),ISNUMBER(O51),ISNUMBER(M51)),((N51/O51)-M51)/(N51/O51),"TBC")</f>
         <v>0.7476923076923078</v>
       </c>
-      <c r="R51" s="1" t="inlineStr">
-        <is>
-          <t>Re:Born Cashmere Fingerless Gloves, Stripes, O/S</t>
-        </is>
-      </c>
+      <c r="R51" s="1" t="n"/>
       <c r="S51" s="1" t="n"/>
       <c r="T51" s="1" t="n"/>
       <c r="U51" s="1" t="n"/>
@@ -5095,13 +4888,13 @@
         <f>"Cashmere "&amp;E52</f>
         <v>Cashmere Reversible Beanie</v>
       </c>
-      <c r="H52" s="35" t="inlineStr">
+      <c r="H52" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
       <c r="I52" t="str">
-        <f>TRIM(MID(R52,FIND(",",R52)+1,FIND(",",R52,FIND(",",R52)+1)-FIND(",",R52)-1))</f>
+        <f>TRIM(MID(K52,FIND(",",K52)+1,FIND(",",K52,FIND(",",K52)+1)-FIND(",",K52)-1))</f>
         <v>Maroon And Dark Brown</v>
       </c>
       <c r="J52" t="inlineStr">
@@ -5109,9 +4902,10 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K52" t="str">
-        <f>VLOOKUP(B52,Lookup!$A$2:$G$7,4,FALSE)&amp;", "&amp;I52&amp;", O/S"</f>
-        <v>Re:Born Reversible Cashmere Beanie, Maroon And Dark Brown, O/S</v>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Re:Born Reversible Cashmere Beanie, Maroon And Dark Brown, O/S</t>
+        </is>
       </c>
       <c r="L52" t="n">
         <v>135</v>
@@ -5135,11 +4929,6 @@
       <c r="Q52">
         <f>IF(AND(ISNUMBER(N52),ISNUMBER(O52),ISNUMBER(M52)),((N52/O52)-M52)/(N52/O52),"TBC")</f>
         <v>0.72</v>
-      </c>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>Re:Born Reverse Cashmere Beanie, Maroon And Dark Brown, O/S</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -5173,37 +4962,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="37" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>Style Code</t>
         </is>
       </c>
-      <c r="B1" s="37" t="inlineStr">
+      <c r="B1" s="36" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="37" t="inlineStr">
+      <c r="C1" s="36" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="D1" s="37" t="inlineStr">
+      <c r="D1" s="36" t="inlineStr">
         <is>
           <t>Brand + Product Name</t>
         </is>
       </c>
-      <c r="E1" s="37" t="inlineStr">
+      <c r="E1" s="36" t="inlineStr">
         <is>
           <t>Cost Price</t>
         </is>
       </c>
-      <c r="F1" s="37" t="inlineStr">
+      <c r="F1" s="36" t="inlineStr">
         <is>
           <t>RRP</t>
         </is>
       </c>
-      <c r="G1" s="37" t="inlineStr">
+      <c r="G1" s="36" t="inlineStr">
         <is>
           <t>Vat</t>
         </is>
@@ -5289,7 +5078,7 @@
       <c r="E4" t="n">
         <v>17.2</v>
       </c>
-      <c r="F4" s="35" t="inlineStr">
+      <c r="F4" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
@@ -5320,7 +5109,7 @@
       <c r="E5" t="n">
         <v>17.2</v>
       </c>
-      <c r="F5" s="35" t="inlineStr">
+      <c r="F5" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
@@ -5348,17 +5137,17 @@
           <t>Re:Born 2 Pack Gloves</t>
         </is>
       </c>
-      <c r="E6" s="35" t="inlineStr">
+      <c r="E6" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="F6" s="35" t="inlineStr">
+      <c r="F6" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="G6" s="35" t="inlineStr">
+      <c r="G6" s="34" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
@@ -5394,21 +5183,21 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="38" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>Style Code = first 6 digits of the Sku.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="38" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>'2 Pack Gloves' has no matching entry on the original ReBorn reference tab - pricing unknown, needs confirming.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="38" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t>RRP for the two 'Set' product lines is shown as '?' on the original ReBorn reference tab - genuinely unconfirmed.</t>
         </is>
@@ -5610,19 +5399,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="38" t="inlineStr">
         <is>
           <t>Re:Born Stock List - Summary Answers</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="40" t="inlineStr">
+      <c r="A3" s="39" t="inlineStr">
         <is>
           <t>Q1. Total stock at net value</t>
         </is>
       </c>
-      <c r="B3" s="41">
+      <c r="B3" s="40">
         <f>SUMPRODUCT(IFERROR('Data Sheet'!P3:P52*'Data Sheet'!L3:L52,0))</f>
         <v>967677.5</v>
       </c>
@@ -5633,24 +5422,24 @@
           <t>Of which, units excluded (price not yet confirmed - see Cleaning Log)</t>
         </is>
       </c>
-      <c r="B4" s="42">
+      <c r="B4" s="41">
         <f>SUMPRODUCT((('Data Sheet'!P3:P52="TBC"))*'Data Sheet'!L3:L52)</f>
         <v>321</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="40" t="inlineStr">
+      <c r="A6" s="39" t="inlineStr">
         <is>
           <t>Q2. Fingerless Gloves currently in stock</t>
         </is>
       </c>
-      <c r="B6" s="42">
+      <c r="B6" s="41">
         <f>SUMIF('Data Sheet'!E3:E52,"Fingerless Gloves",'Data Sheet'!L3:L52)</f>
         <v>29118</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="40" t="inlineStr">
+      <c r="A8" s="39" t="inlineStr">
         <is>
           <t>Stock quantity by category (reference)</t>
         </is>
@@ -5662,7 +5451,7 @@
           <t>Fingerless Gloves</t>
         </is>
       </c>
-      <c r="B9" s="42">
+      <c r="B9" s="41">
         <f>SUMIF('Data Sheet'!E3:E52,"Fingerless Gloves",'Data Sheet'!L3:L52)</f>
         <v>29118</v>
       </c>
@@ -5673,7 +5462,7 @@
           <t>Reversible Beanie</t>
         </is>
       </c>
-      <c r="B10" s="42">
+      <c r="B10" s="41">
         <f>SUMIF('Data Sheet'!E3:E52,"Reversible Beanie",'Data Sheet'!L3:L52)</f>
         <v>241</v>
       </c>
@@ -5684,7 +5473,7 @@
           <t>Reversible Snood</t>
         </is>
       </c>
-      <c r="B11" s="42">
+      <c r="B11" s="41">
         <f>SUMIF('Data Sheet'!E3:E52,"Reversible Snood",'Data Sheet'!L3:L52)</f>
         <v>386</v>
       </c>
@@ -5695,7 +5484,7 @@
           <t>Snood &amp; Glove Set</t>
         </is>
       </c>
-      <c r="B12" s="42">
+      <c r="B12" s="41">
         <f>SUMIF('Data Sheet'!E3:E52,"Snood &amp; Glove Set",'Data Sheet'!L3:L52)</f>
         <v>35</v>
       </c>
@@ -5706,7 +5495,7 @@
           <t>Beanie &amp; Glove Set</t>
         </is>
       </c>
-      <c r="B13" s="42">
+      <c r="B13" s="41">
         <f>SUMIF('Data Sheet'!E3:E52,"Beanie &amp; Glove Set",'Data Sheet'!L3:L52)</f>
         <v>147</v>
       </c>
@@ -5717,13 +5506,13 @@
           <t>2 Pack Gloves</t>
         </is>
       </c>
-      <c r="B14" s="42">
+      <c r="B14" s="41">
         <f>SUMIF('Data Sheet'!E3:E52,"2 Pack Gloves",'Data Sheet'!L3:L52)</f>
         <v>139</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="40" t="inlineStr">
+      <c r="A16" s="39" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
@@ -5781,447 +5570,447 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="38" t="inlineStr">
         <is>
           <t>Data Cleaning Log - Re:Born Stock List</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="37" t="inlineStr">
+      <c r="A3" s="36" t="inlineStr">
         <is>
           <t>Original Row(s)</t>
         </is>
       </c>
-      <c r="B3" s="37" t="inlineStr">
+      <c r="B3" s="36" t="inlineStr">
         <is>
           <t>Issue Found</t>
         </is>
       </c>
-      <c r="C3" s="37" t="inlineStr">
+      <c r="C3" s="36" t="inlineStr">
         <is>
           <t>Resolution</t>
         </is>
       </c>
-      <c r="D3" s="37" t="inlineStr">
+      <c r="D3" s="36" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="43" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr">
         <is>
           <t>Row 41</t>
         </is>
       </c>
-      <c r="B4" s="43" t="inlineStr">
+      <c r="B4" s="42" t="inlineStr">
         <is>
           <t>Completely blank row in the middle of the sheet.</t>
         </is>
       </c>
-      <c r="C4" s="43" t="inlineStr">
+      <c r="C4" s="42" t="inlineStr">
         <is>
           <t>Row removed.</t>
         </is>
       </c>
-      <c r="D4" s="43" t="inlineStr">
+      <c r="D4" s="42" t="inlineStr">
         <is>
           <t>Blank row</t>
         </is>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="43" t="inlineStr">
+      <c r="A5" s="42" t="inlineStr">
         <is>
           <t>Rows 4 &amp; 5</t>
         </is>
       </c>
-      <c r="B5" s="43" t="inlineStr">
+      <c r="B5" s="42" t="inlineStr">
         <is>
           <t>Sku 900236ZZLGRY0000 listed twice with identical qty (3605) and identical description.</t>
         </is>
       </c>
-      <c r="C5" s="43" t="inlineStr">
+      <c r="C5" s="42" t="inlineStr">
         <is>
           <t>Kept row 4, removed the exact duplicate.</t>
         </is>
       </c>
-      <c r="D5" s="43" t="inlineStr">
+      <c r="D5" s="42" t="inlineStr">
         <is>
           <t>Exact duplicate</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="43" t="inlineStr">
+      <c r="A6" s="42" t="inlineStr">
         <is>
           <t>Rows 6 &amp; 7</t>
         </is>
       </c>
-      <c r="B6" s="43" t="inlineStr">
+      <c r="B6" s="42" t="inlineStr">
         <is>
           <t>Sku 900236ZZDKGR0000 listed twice with identical qty (3599) and identical description.</t>
         </is>
       </c>
-      <c r="C6" s="43" t="inlineStr">
+      <c r="C6" s="42" t="inlineStr">
         <is>
           <t>Kept row 6, removed the exact duplicate.</t>
         </is>
       </c>
-      <c r="D6" s="43" t="inlineStr">
+      <c r="D6" s="42" t="inlineStr">
         <is>
           <t>Exact duplicate</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="43" t="inlineStr">
+      <c r="A7" s="42" t="inlineStr">
         <is>
           <t>Rows 58 &amp; 59</t>
         </is>
       </c>
-      <c r="B7" s="43" t="inlineStr">
+      <c r="B7" s="42" t="inlineStr">
         <is>
           <t>Sku 900236ZZAAAI0000 (Teal) listed twice with identical qty (138) and identical description.</t>
         </is>
       </c>
-      <c r="C7" s="43" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
         <is>
           <t>Kept row 58, removed the exact duplicate.</t>
         </is>
       </c>
-      <c r="D7" s="43" t="inlineStr">
+      <c r="D7" s="42" t="inlineStr">
         <is>
           <t>Exact duplicate</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="43" t="inlineStr">
+      <c r="A8" s="42" t="inlineStr">
         <is>
           <t>Rows 17 &amp; 18</t>
         </is>
       </c>
-      <c r="B8" s="43" t="inlineStr">
+      <c r="B8" s="42" t="inlineStr">
         <is>
           <t>Sku 900236ZZDMAA0000 listed twice, same qty (598), but row 18's description drops the word 'Fingerless' and uses 'One Size' instead of 'O/S'.</t>
         </is>
       </c>
-      <c r="C8" s="43" t="inlineStr">
+      <c r="C8" s="42" t="inlineStr">
         <is>
           <t>Kept row 17 (matches the standard description format used everywhere else), removed row 18.</t>
         </is>
       </c>
-      <c r="D8" s="43" t="inlineStr">
+      <c r="D8" s="42" t="inlineStr">
         <is>
           <t>Duplicate - inconsistent wording</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="43" t="inlineStr">
+      <c r="A9" s="42" t="inlineStr">
         <is>
           <t>Rows 30 &amp; 31</t>
         </is>
       </c>
-      <c r="B9" s="43" t="inlineStr">
+      <c r="B9" s="42" t="inlineStr">
         <is>
           <t>Sku 900235ZZBCAA0000 listed twice, same qty (41); row 31 spells the brand 'RE:Born' (wrong capitalisation) instead of 'Re:Born'.</t>
         </is>
       </c>
-      <c r="C9" s="43" t="inlineStr">
+      <c r="C9" s="42" t="inlineStr">
         <is>
           <t>Kept row 30, removed the typo duplicate.</t>
         </is>
       </c>
-      <c r="D9" s="43" t="inlineStr">
+      <c r="D9" s="42" t="inlineStr">
         <is>
           <t>Duplicate - typo</t>
         </is>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="43" t="inlineStr">
+      <c r="A10" s="42" t="inlineStr">
         <is>
           <t>Rows 36 &amp; 47</t>
         </is>
       </c>
-      <c r="B10" s="43" t="inlineStr">
+      <c r="B10" s="42" t="inlineStr">
         <is>
           <t>Sku 900232ZZBGAA0000 listed twice (not adjacent - easy to miss), same qty (11); row 36 has a double space and is 8 rows away from its duplicate at row 47.</t>
         </is>
       </c>
-      <c r="C10" s="43" t="inlineStr">
+      <c r="C10" s="42" t="inlineStr">
         <is>
           <t>Kept row 47, removed row 36.</t>
         </is>
       </c>
-      <c r="D10" s="43" t="inlineStr">
+      <c r="D10" s="42" t="inlineStr">
         <is>
           <t>Duplicate - formatting/typo, non-adjacent</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="A11" s="42" t="inlineStr">
         <is>
           <t>Rows 37 &amp; 38</t>
         </is>
       </c>
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B11" s="42" t="inlineStr">
         <is>
           <t>Sku 900231ZZBLLL0000 listed twice, same qty (11); row 37 drops the word 'Cashmere' and has a double space.</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>Kept row 38, removed row 37.</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="42" t="inlineStr">
         <is>
           <t>Duplicate - inconsistent wording</t>
         </is>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="43" t="inlineStr">
+      <c r="A12" s="42" t="inlineStr">
         <is>
           <t>Rows 43 &amp; 53</t>
         </is>
       </c>
-      <c r="B12" s="43" t="inlineStr">
+      <c r="B12" s="42" t="inlineStr">
         <is>
           <t>Sku 900231ZZBPAA0000 listed twice, same qty (49), 10 rows apart; row 53 misspells the brand as 'Re:Bron'.</t>
         </is>
       </c>
-      <c r="C12" s="43" t="inlineStr">
+      <c r="C12" s="42" t="inlineStr">
         <is>
           <t>Kept row 43, removed row 53.</t>
         </is>
       </c>
-      <c r="D12" s="43" t="inlineStr">
+      <c r="D12" s="42" t="inlineStr">
         <is>
           <t>Duplicate - typo, non-adjacent</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="43" t="inlineStr">
+      <c r="A13" s="42" t="inlineStr">
         <is>
           <t>All Reversible Beanie rows</t>
         </is>
       </c>
-      <c r="B13" s="43" t="inlineStr">
+      <c r="B13" s="42" t="inlineStr">
         <is>
           <t>Product name inconsistently written as 'Reverse Beanie' / 'Reverse Cashmere Beanie' in some rows vs 'Reversible Cashmere Beanie' in others. The ReBorn reference tab confirms 'Reversible' is correct.</t>
         </is>
       </c>
-      <c r="C13" s="43" t="inlineStr">
+      <c r="C13" s="42" t="inlineStr">
         <is>
           <t>Standardised every row's Description to 'Re:Born Reversible Cashmere Beanie, &lt;colour&gt;, O/S'.</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
+      <c r="D13" s="42" t="inlineStr">
         <is>
           <t>Inconsistent naming</t>
         </is>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="43" t="inlineStr">
+      <c r="A14" s="42" t="inlineStr">
         <is>
           <t>Style Code / Colour Code / Option (cols B-D)</t>
         </is>
       </c>
-      <c r="B14" s="43" t="inlineStr">
+      <c r="B14" s="42" t="inlineStr">
         <is>
           <t>Not filled in for any row except the example (row 2). Also, row 2's own Option (900196AUBE) does not actually match its own Style Code (900000) or Sku - the example itself contains an inconsistency.</t>
         </is>
       </c>
-      <c r="C14" s="43" t="inlineStr">
+      <c r="C14" s="42" t="inlineStr">
         <is>
           <t>Derived Style Code and Colour Code directly from each Sku (first 6 digits / the 4 letters between 'ZZ' and the trailing '0000'), and built Option as Style Code + Colour Code consistently for every row.</t>
         </is>
       </c>
-      <c r="D14" s="43" t="inlineStr">
+      <c r="D14" s="42" t="inlineStr">
         <is>
           <t>Missing data + example inconsistency</t>
         </is>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="43" t="inlineStr">
+      <c r="A15" s="42" t="inlineStr">
         <is>
           <t>Category / Material / Style (cols E-G)</t>
         </is>
       </c>
-      <c r="B15" s="43" t="inlineStr">
+      <c r="B15" s="42" t="inlineStr">
         <is>
           <t>Not filled in for any row.</t>
         </is>
       </c>
-      <c r="C15" s="43" t="inlineStr">
+      <c r="C15" s="42" t="inlineStr">
         <is>
           <t>Derived from the 6-digit style-code prefix of the Sku (e.g. 900236 = Fingerless Gloves), cross-checked against the product names on the ReBorn reference tab.</t>
         </is>
       </c>
-      <c r="D15" s="43" t="inlineStr">
+      <c r="D15" s="42" t="inlineStr">
         <is>
           <t>Missing data</t>
         </is>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="43" t="inlineStr">
+      <c r="A16" s="42" t="inlineStr">
         <is>
           <t>Colour (col I)</t>
         </is>
       </c>
-      <c r="B16" s="43" t="inlineStr">
+      <c r="B16" s="42" t="inlineStr">
         <is>
           <t>Not filled in for any row.</t>
         </is>
       </c>
-      <c r="C16" s="43" t="inlineStr">
+      <c r="C16" s="42" t="inlineStr">
         <is>
           <t>Extracted from the middle segment of each Description (text between the two commas).</t>
         </is>
       </c>
-      <c r="D16" s="43" t="inlineStr">
+      <c r="D16" s="42" t="inlineStr">
         <is>
           <t>Missing data</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="43" t="inlineStr">
+      <c r="A17" s="42" t="inlineStr">
         <is>
           <t>Size (col J)</t>
         </is>
       </c>
-      <c r="B17" s="43" t="inlineStr">
+      <c r="B17" s="42" t="inlineStr">
         <is>
           <t>Not filled in for any row.</t>
         </is>
       </c>
-      <c r="C17" s="43" t="inlineStr">
+      <c r="C17" s="42" t="inlineStr">
         <is>
           <t>Set to 'One Size' for every row - every product in this list is O/S (one size).</t>
         </is>
       </c>
-      <c r="D17" s="43" t="inlineStr">
+      <c r="D17" s="42" t="inlineStr">
         <is>
           <t>Missing data</t>
         </is>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="43" t="inlineStr">
+      <c r="A18" s="42" t="inlineStr">
         <is>
           <t>Landed Cost Price / RRP / Vat (cols M-O)</t>
         </is>
       </c>
-      <c r="B18" s="43" t="inlineStr">
+      <c r="B18" s="42" t="inlineStr">
         <is>
           <t>Not filled in for any row.</t>
         </is>
       </c>
-      <c r="C18" s="43" t="inlineStr">
+      <c r="C18" s="42" t="inlineStr">
         <is>
           <t>Looked up from the ReBorn reference tab by product category and applied to every row in that category.</t>
         </is>
       </c>
-      <c r="D18" s="43" t="inlineStr">
+      <c r="D18" s="42" t="inlineStr">
         <is>
           <t>Missing data</t>
         </is>
       </c>
     </row>
     <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="43" t="inlineStr">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>Net RRP / Margin (cols P-Q)</t>
         </is>
       </c>
-      <c r="B19" s="43" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t>Not filled in for any row.</t>
         </is>
       </c>
-      <c r="C19" s="43" t="inlineStr">
+      <c r="C19" s="42" t="inlineStr">
         <is>
           <t>Copied the same formulas used in the row 2 example (Net RRP = RRP/Vat, Margin = (Net RRP - Cost)/Net RRP) down every row where RRP is known.</t>
         </is>
       </c>
-      <c r="D19" s="43" t="inlineStr">
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>Missing data</t>
         </is>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="43" t="inlineStr">
+      <c r="A20" s="42" t="inlineStr">
         <is>
           <t>2 Pack Gloves pricing (style 900235)</t>
         </is>
       </c>
-      <c r="B20" s="43" t="inlineStr">
+      <c r="B20" s="42" t="inlineStr">
         <is>
           <t>This product line (several rows) has no matching entry anywhere on the ReBorn reference tab, so Cost Price, RRP and Vat are all unknown.</t>
         </is>
       </c>
-      <c r="C20" s="43" t="inlineStr">
+      <c r="C20" s="42" t="inlineStr">
         <is>
           <t>Left marked 'TBC' (highlighted) in Cost Price, RRP, Vat, Net RRP and Margin. Recommend checking with the buying/finance team for the correct figures.</t>
         </is>
       </c>
-      <c r="D20" s="43" t="inlineStr">
+      <c r="D20" s="42" t="inlineStr">
         <is>
           <t>Further investigation needed</t>
         </is>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="43" t="inlineStr">
+      <c r="A21" s="42" t="inlineStr">
         <is>
           <t>Snood &amp; Glove Set / Beanie &amp; Glove Set RRP</t>
         </is>
       </c>
-      <c r="B21" s="43" t="inlineStr">
+      <c r="B21" s="42" t="inlineStr">
         <is>
           <t>The ReBorn reference tab lists the RRP for these two lines as '?' - i.e. genuinely not yet decided/confirmed, not a data entry gap.</t>
         </is>
       </c>
-      <c r="C21" s="43" t="inlineStr">
+      <c r="C21" s="42" t="inlineStr">
         <is>
           <t>Cost Price and Vat filled in from the reference tab; RRP, Net RRP and Margin left as 'TBC' (highlighted) since inventing a number would be misleading. Recommend confirming with pricing/marketing.</t>
         </is>
       </c>
-      <c r="D21" s="43" t="inlineStr">
+      <c r="D21" s="42" t="inlineStr">
         <is>
           <t>Further investigation needed</t>
         </is>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="43" t="inlineStr">
+      <c r="A22" s="42" t="inlineStr">
         <is>
           <t>Range (col H)</t>
         </is>
       </c>
-      <c r="B22" s="43" t="inlineStr">
+      <c r="B22" s="42" t="inlineStr">
         <is>
           <t>The row 2 example shows a Range of 'Core', but no other row, sheet, or column in the source data indicates what Range/Collection any product belongs to.</t>
         </is>
       </c>
-      <c r="C22" s="43" t="inlineStr">
+      <c r="C22" s="42" t="inlineStr">
         <is>
           <t>Left as 'TBC' (highlighted) for every row rather than guessing. Recommend checking with merchandising for the correct Range per style.</t>
         </is>
       </c>
-      <c r="D22" s="43" t="inlineStr">
+      <c r="D22" s="42" t="inlineStr">
         <is>
           <t>Further investigation needed</t>
         </is>

</xml_diff>

<commit_message>
Apply wrap-text formatting to Description column for all rows
Row 2 (the original example) had "Wrap Text" enabled on its
Description cell; every other row didn't, so the full text was
truncated instead of wrapping within the cell. Applied the same
formatting to the Description column across all rows.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192FU3Scg9XSr7HEGSJ8k2R
</commit_message>
<xml_diff>
--- a/ReBorn_stock_list_26_FINAL.xlsx
+++ b/ReBorn_stock_list_26_FINAL.xlsx
@@ -153,7 +153,7 @@
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,6 +223,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="4"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1125,7 +1128,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Black, O/S</t>
         </is>
@@ -1198,7 +1201,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Light Grey, O/S</t>
         </is>
@@ -1271,7 +1274,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Dark Grey, O/S</t>
         </is>
@@ -1344,7 +1347,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Light Beige, O/S</t>
         </is>
@@ -1417,7 +1420,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K7" s="27" t="inlineStr">
+      <c r="K7" s="35" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Light Brown, O/S</t>
         </is>
@@ -1476,7 +1479,7 @@
         <f>"Cashmere "&amp;E8</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H8" s="35" t="inlineStr">
+      <c r="H8" s="36" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
@@ -1490,7 +1493,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Navy, O/S</t>
         </is>
@@ -1603,7 +1606,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K9" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Light Maroon, O/S</t>
         </is>
@@ -1662,7 +1665,7 @@
         <f>"Cashmere "&amp;E10</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H10" s="35" t="inlineStr">
+      <c r="H10" s="36" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
@@ -1676,7 +1679,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K10" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Red, O/S</t>
         </is>
@@ -1789,7 +1792,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Baby Pink, O/S</t>
         </is>
@@ -1862,7 +1865,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K12" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Dark Brown, O/S</t>
         </is>
@@ -1935,7 +1938,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Yellow, O/S</t>
         </is>
@@ -2008,7 +2011,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K14" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Beige, O/S</t>
         </is>
@@ -2081,7 +2084,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K15" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Deep Matcha Green, O/S</t>
         </is>
@@ -2154,7 +2157,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K16" s="26" t="inlineStr">
+      <c r="K16" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Pink, O/S</t>
         </is>
@@ -2227,7 +2230,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K17" s="26" t="inlineStr">
+      <c r="K17" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Military Green, O/S</t>
         </is>
@@ -2300,7 +2303,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K18" s="26" t="inlineStr">
+      <c r="K18" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Light Green, O/S</t>
         </is>
@@ -2373,7 +2376,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K19" s="26" t="inlineStr">
+      <c r="K19" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Light Blue, O/S</t>
         </is>
@@ -2446,7 +2449,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K20" s="26" t="inlineStr">
+      <c r="K20" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Lavender, O/S</t>
         </is>
@@ -2519,7 +2522,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K21" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Maroon, O/S</t>
         </is>
@@ -2592,7 +2595,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K22" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Denim Blue, O/S</t>
         </is>
@@ -2665,7 +2668,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K23" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Kelly Green, O/S</t>
         </is>
@@ -2738,7 +2741,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K24" s="14" t="inlineStr">
         <is>
           <t>Re:Born Beanie &amp; Glove Set, Black &amp; Red, O/S</t>
         </is>
@@ -2811,7 +2814,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="K25" s="14" t="inlineStr">
         <is>
           <t>Re:Born 2 Pack Gloves, Red And Navy, O/S</t>
         </is>
@@ -2884,7 +2887,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Hot Pink, O/S</t>
         </is>
@@ -2957,7 +2960,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" s="14" t="inlineStr">
         <is>
           <t>Re:Born 2 Pack Gloves, Black And Caramel, O/S</t>
         </is>
@@ -3030,7 +3033,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K28" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, One Of A Kind, O/S</t>
         </is>
@@ -3103,7 +3106,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K29" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Brights, O/S</t>
         </is>
@@ -3176,7 +3179,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K30" s="14" t="inlineStr">
         <is>
           <t>Re:Born Beanie &amp; Glove Set, Navy And Beige, O/S</t>
         </is>
@@ -3249,7 +3252,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K31" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Beanie, Light Blue&amp;Light Beige, O/S</t>
         </is>
@@ -3322,7 +3325,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K32" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Beanie, Black And Light Grey, O/S</t>
         </is>
@@ -3395,7 +3398,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Orange, O/S</t>
         </is>
@@ -3454,7 +3457,7 @@
         <f>"Cashmere "&amp;E34</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H34" s="35" t="inlineStr">
+      <c r="H34" s="36" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
@@ -3468,7 +3471,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K34" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Royal Blue, O/S</t>
         </is>
@@ -3581,7 +3584,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="K35" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Snood, Light Beige&amp;Choco Brown, O/S</t>
         </is>
@@ -3654,7 +3657,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K36" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Beanie, Baby Pink And Cream, O/S</t>
         </is>
@@ -3727,7 +3730,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K37" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Beanie, Purple And Yellow, O/S</t>
         </is>
@@ -3800,7 +3803,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="K38" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Beanie, Red And Beige, O/S</t>
         </is>
@@ -3873,7 +3876,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K39" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Snood, Beige And Brown, O/S</t>
         </is>
@@ -3946,7 +3949,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="K40" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Snood, Black And Dark Grey, O/S</t>
         </is>
@@ -4019,7 +4022,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Snood, Black, O/S</t>
         </is>
@@ -4092,7 +4095,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K42" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Snood, Light Grey And Black, O/S</t>
         </is>
@@ -4165,7 +4168,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Snood, Maroon And Dark Grey, O/S</t>
         </is>
@@ -4238,7 +4241,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K44" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Snood, Red And Cream, O/S</t>
         </is>
@@ -4311,7 +4314,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="14" t="inlineStr">
         <is>
           <t>Re:Born Snood &amp; Glove Set, Navy/Red and Grey, O/S</t>
         </is>
@@ -4384,7 +4387,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K46" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Grape Purple, O/S</t>
         </is>
@@ -4457,7 +4460,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K47" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Dark Purple, O/S</t>
         </is>
@@ -4516,7 +4519,7 @@
         <f>"Cashmere "&amp;E48</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H48" s="35" t="inlineStr">
+      <c r="H48" s="36" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
@@ -4530,7 +4533,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K48" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Ocean Green, O/S</t>
         </is>
@@ -4643,7 +4646,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K49" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Baby Blue, O/S</t>
         </is>
@@ -4716,7 +4719,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="K50" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Teal, O/S</t>
         </is>
@@ -4775,7 +4778,7 @@
         <f>"Cashmere "&amp;E51</f>
         <v>Cashmere Fingerless Gloves</v>
       </c>
-      <c r="H51" s="35" t="inlineStr">
+      <c r="H51" s="36" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
@@ -4789,7 +4792,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
+      <c r="K51" s="14" t="inlineStr">
         <is>
           <t>Re:Born Cashmere Fingerless Gloves, Stripes, O/S</t>
         </is>
@@ -4902,7 +4905,7 @@
           <t>One Size</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="K52" s="14" t="inlineStr">
         <is>
           <t>Re:Born Reversible Cashmere Beanie, Maroon And Dark Brown, O/S</t>
         </is>
@@ -4962,37 +4965,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="36" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Style Code</t>
         </is>
       </c>
-      <c r="B1" s="36" t="inlineStr">
+      <c r="B1" s="37" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="36" t="inlineStr">
+      <c r="C1" s="37" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="D1" s="36" t="inlineStr">
+      <c r="D1" s="37" t="inlineStr">
         <is>
           <t>Brand + Product Name</t>
         </is>
       </c>
-      <c r="E1" s="36" t="inlineStr">
+      <c r="E1" s="37" t="inlineStr">
         <is>
           <t>Cost Price</t>
         </is>
       </c>
-      <c r="F1" s="36" t="inlineStr">
+      <c r="F1" s="37" t="inlineStr">
         <is>
           <t>RRP</t>
         </is>
       </c>
-      <c r="G1" s="36" t="inlineStr">
+      <c r="G1" s="37" t="inlineStr">
         <is>
           <t>Vat</t>
         </is>
@@ -5183,21 +5186,21 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="37" t="inlineStr">
+      <c r="A9" s="38" t="inlineStr">
         <is>
           <t>Style Code = first 6 digits of the Sku.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="37" t="inlineStr">
+      <c r="A10" s="38" t="inlineStr">
         <is>
           <t>'2 Pack Gloves' has no matching entry on the original ReBorn reference tab - pricing unknown, needs confirming.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="37" t="inlineStr">
+      <c r="A11" s="38" t="inlineStr">
         <is>
           <t>RRP for the two 'Set' product lines is shown as '?' on the original ReBorn reference tab - genuinely unconfirmed.</t>
         </is>
@@ -5399,19 +5402,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="39" t="inlineStr">
         <is>
           <t>Re:Born Stock List - Summary Answers</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="39" t="inlineStr">
+      <c r="A3" s="40" t="inlineStr">
         <is>
           <t>Q1. Total stock at net value</t>
         </is>
       </c>
-      <c r="B3" s="40">
+      <c r="B3" s="41">
         <f>SUMPRODUCT(IFERROR('Data Sheet'!P3:P52*'Data Sheet'!L3:L52,0))</f>
         <v>967677.5</v>
       </c>
@@ -5422,24 +5425,24 @@
           <t>Of which, units excluded (price not yet confirmed - see Cleaning Log)</t>
         </is>
       </c>
-      <c r="B4" s="41">
+      <c r="B4" s="42">
         <f>SUMPRODUCT((('Data Sheet'!P3:P52="TBC"))*'Data Sheet'!L3:L52)</f>
         <v>321</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="39" t="inlineStr">
+      <c r="A6" s="40" t="inlineStr">
         <is>
           <t>Q2. Fingerless Gloves currently in stock</t>
         </is>
       </c>
-      <c r="B6" s="41">
+      <c r="B6" s="42">
         <f>SUMIF('Data Sheet'!E3:E52,"Fingerless Gloves",'Data Sheet'!L3:L52)</f>
         <v>29118</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="40" t="inlineStr">
         <is>
           <t>Stock quantity by category (reference)</t>
         </is>
@@ -5451,7 +5454,7 @@
           <t>Fingerless Gloves</t>
         </is>
       </c>
-      <c r="B9" s="41">
+      <c r="B9" s="42">
         <f>SUMIF('Data Sheet'!E3:E52,"Fingerless Gloves",'Data Sheet'!L3:L52)</f>
         <v>29118</v>
       </c>
@@ -5462,7 +5465,7 @@
           <t>Reversible Beanie</t>
         </is>
       </c>
-      <c r="B10" s="41">
+      <c r="B10" s="42">
         <f>SUMIF('Data Sheet'!E3:E52,"Reversible Beanie",'Data Sheet'!L3:L52)</f>
         <v>241</v>
       </c>
@@ -5473,7 +5476,7 @@
           <t>Reversible Snood</t>
         </is>
       </c>
-      <c r="B11" s="41">
+      <c r="B11" s="42">
         <f>SUMIF('Data Sheet'!E3:E52,"Reversible Snood",'Data Sheet'!L3:L52)</f>
         <v>386</v>
       </c>
@@ -5484,7 +5487,7 @@
           <t>Snood &amp; Glove Set</t>
         </is>
       </c>
-      <c r="B12" s="41">
+      <c r="B12" s="42">
         <f>SUMIF('Data Sheet'!E3:E52,"Snood &amp; Glove Set",'Data Sheet'!L3:L52)</f>
         <v>35</v>
       </c>
@@ -5495,7 +5498,7 @@
           <t>Beanie &amp; Glove Set</t>
         </is>
       </c>
-      <c r="B13" s="41">
+      <c r="B13" s="42">
         <f>SUMIF('Data Sheet'!E3:E52,"Beanie &amp; Glove Set",'Data Sheet'!L3:L52)</f>
         <v>147</v>
       </c>
@@ -5506,13 +5509,13 @@
           <t>2 Pack Gloves</t>
         </is>
       </c>
-      <c r="B14" s="41">
+      <c r="B14" s="42">
         <f>SUMIF('Data Sheet'!E3:E52,"2 Pack Gloves",'Data Sheet'!L3:L52)</f>
         <v>139</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="39" t="inlineStr">
+      <c r="A16" s="40" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
@@ -5570,447 +5573,447 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="39" t="inlineStr">
         <is>
           <t>Data Cleaning Log - Re:Born Stock List</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="36" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
         <is>
           <t>Original Row(s)</t>
         </is>
       </c>
-      <c r="B3" s="36" t="inlineStr">
+      <c r="B3" s="37" t="inlineStr">
         <is>
           <t>Issue Found</t>
         </is>
       </c>
-      <c r="C3" s="36" t="inlineStr">
+      <c r="C3" s="37" t="inlineStr">
         <is>
           <t>Resolution</t>
         </is>
       </c>
-      <c r="D3" s="36" t="inlineStr">
+      <c r="D3" s="37" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="A4" s="43" t="inlineStr">
         <is>
           <t>Row 41</t>
         </is>
       </c>
-      <c r="B4" s="42" t="inlineStr">
+      <c r="B4" s="43" t="inlineStr">
         <is>
           <t>Completely blank row in the middle of the sheet.</t>
         </is>
       </c>
-      <c r="C4" s="42" t="inlineStr">
+      <c r="C4" s="43" t="inlineStr">
         <is>
           <t>Row removed.</t>
         </is>
       </c>
-      <c r="D4" s="42" t="inlineStr">
+      <c r="D4" s="43" t="inlineStr">
         <is>
           <t>Blank row</t>
         </is>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="42" t="inlineStr">
+      <c r="A5" s="43" t="inlineStr">
         <is>
           <t>Rows 4 &amp; 5</t>
         </is>
       </c>
-      <c r="B5" s="42" t="inlineStr">
+      <c r="B5" s="43" t="inlineStr">
         <is>
           <t>Sku 900236ZZLGRY0000 listed twice with identical qty (3605) and identical description.</t>
         </is>
       </c>
-      <c r="C5" s="42" t="inlineStr">
+      <c r="C5" s="43" t="inlineStr">
         <is>
           <t>Kept row 4, removed the exact duplicate.</t>
         </is>
       </c>
-      <c r="D5" s="42" t="inlineStr">
+      <c r="D5" s="43" t="inlineStr">
         <is>
           <t>Exact duplicate</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="42" t="inlineStr">
+      <c r="A6" s="43" t="inlineStr">
         <is>
           <t>Rows 6 &amp; 7</t>
         </is>
       </c>
-      <c r="B6" s="42" t="inlineStr">
+      <c r="B6" s="43" t="inlineStr">
         <is>
           <t>Sku 900236ZZDKGR0000 listed twice with identical qty (3599) and identical description.</t>
         </is>
       </c>
-      <c r="C6" s="42" t="inlineStr">
+      <c r="C6" s="43" t="inlineStr">
         <is>
           <t>Kept row 6, removed the exact duplicate.</t>
         </is>
       </c>
-      <c r="D6" s="42" t="inlineStr">
+      <c r="D6" s="43" t="inlineStr">
         <is>
           <t>Exact duplicate</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="42" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Rows 58 &amp; 59</t>
         </is>
       </c>
-      <c r="B7" s="42" t="inlineStr">
+      <c r="B7" s="43" t="inlineStr">
         <is>
           <t>Sku 900236ZZAAAI0000 (Teal) listed twice with identical qty (138) and identical description.</t>
         </is>
       </c>
-      <c r="C7" s="42" t="inlineStr">
+      <c r="C7" s="43" t="inlineStr">
         <is>
           <t>Kept row 58, removed the exact duplicate.</t>
         </is>
       </c>
-      <c r="D7" s="42" t="inlineStr">
+      <c r="D7" s="43" t="inlineStr">
         <is>
           <t>Exact duplicate</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="42" t="inlineStr">
+      <c r="A8" s="43" t="inlineStr">
         <is>
           <t>Rows 17 &amp; 18</t>
         </is>
       </c>
-      <c r="B8" s="42" t="inlineStr">
+      <c r="B8" s="43" t="inlineStr">
         <is>
           <t>Sku 900236ZZDMAA0000 listed twice, same qty (598), but row 18's description drops the word 'Fingerless' and uses 'One Size' instead of 'O/S'.</t>
         </is>
       </c>
-      <c r="C8" s="42" t="inlineStr">
+      <c r="C8" s="43" t="inlineStr">
         <is>
           <t>Kept row 17 (matches the standard description format used everywhere else), removed row 18.</t>
         </is>
       </c>
-      <c r="D8" s="42" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
         <is>
           <t>Duplicate - inconsistent wording</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="42" t="inlineStr">
+      <c r="A9" s="43" t="inlineStr">
         <is>
           <t>Rows 30 &amp; 31</t>
         </is>
       </c>
-      <c r="B9" s="42" t="inlineStr">
+      <c r="B9" s="43" t="inlineStr">
         <is>
           <t>Sku 900235ZZBCAA0000 listed twice, same qty (41); row 31 spells the brand 'RE:Born' (wrong capitalisation) instead of 'Re:Born'.</t>
         </is>
       </c>
-      <c r="C9" s="42" t="inlineStr">
+      <c r="C9" s="43" t="inlineStr">
         <is>
           <t>Kept row 30, removed the typo duplicate.</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
+      <c r="D9" s="43" t="inlineStr">
         <is>
           <t>Duplicate - typo</t>
         </is>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="42" t="inlineStr">
+      <c r="A10" s="43" t="inlineStr">
         <is>
           <t>Rows 36 &amp; 47</t>
         </is>
       </c>
-      <c r="B10" s="42" t="inlineStr">
+      <c r="B10" s="43" t="inlineStr">
         <is>
           <t>Sku 900232ZZBGAA0000 listed twice (not adjacent - easy to miss), same qty (11); row 36 has a double space and is 8 rows away from its duplicate at row 47.</t>
         </is>
       </c>
-      <c r="C10" s="42" t="inlineStr">
+      <c r="C10" s="43" t="inlineStr">
         <is>
           <t>Kept row 47, removed row 36.</t>
         </is>
       </c>
-      <c r="D10" s="42" t="inlineStr">
+      <c r="D10" s="43" t="inlineStr">
         <is>
           <t>Duplicate - formatting/typo, non-adjacent</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="42" t="inlineStr">
+      <c r="A11" s="43" t="inlineStr">
         <is>
           <t>Rows 37 &amp; 38</t>
         </is>
       </c>
-      <c r="B11" s="42" t="inlineStr">
+      <c r="B11" s="43" t="inlineStr">
         <is>
           <t>Sku 900231ZZBLLL0000 listed twice, same qty (11); row 37 drops the word 'Cashmere' and has a double space.</t>
         </is>
       </c>
-      <c r="C11" s="42" t="inlineStr">
+      <c r="C11" s="43" t="inlineStr">
         <is>
           <t>Kept row 38, removed row 37.</t>
         </is>
       </c>
-      <c r="D11" s="42" t="inlineStr">
+      <c r="D11" s="43" t="inlineStr">
         <is>
           <t>Duplicate - inconsistent wording</t>
         </is>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="42" t="inlineStr">
+      <c r="A12" s="43" t="inlineStr">
         <is>
           <t>Rows 43 &amp; 53</t>
         </is>
       </c>
-      <c r="B12" s="42" t="inlineStr">
+      <c r="B12" s="43" t="inlineStr">
         <is>
           <t>Sku 900231ZZBPAA0000 listed twice, same qty (49), 10 rows apart; row 53 misspells the brand as 'Re:Bron'.</t>
         </is>
       </c>
-      <c r="C12" s="42" t="inlineStr">
+      <c r="C12" s="43" t="inlineStr">
         <is>
           <t>Kept row 43, removed row 53.</t>
         </is>
       </c>
-      <c r="D12" s="42" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>Duplicate - typo, non-adjacent</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="42" t="inlineStr">
+      <c r="A13" s="43" t="inlineStr">
         <is>
           <t>All Reversible Beanie rows</t>
         </is>
       </c>
-      <c r="B13" s="42" t="inlineStr">
+      <c r="B13" s="43" t="inlineStr">
         <is>
           <t>Product name inconsistently written as 'Reverse Beanie' / 'Reverse Cashmere Beanie' in some rows vs 'Reversible Cashmere Beanie' in others. The ReBorn reference tab confirms 'Reversible' is correct.</t>
         </is>
       </c>
-      <c r="C13" s="42" t="inlineStr">
+      <c r="C13" s="43" t="inlineStr">
         <is>
           <t>Standardised every row's Description to 'Re:Born Reversible Cashmere Beanie, &lt;colour&gt;, O/S'.</t>
         </is>
       </c>
-      <c r="D13" s="42" t="inlineStr">
+      <c r="D13" s="43" t="inlineStr">
         <is>
           <t>Inconsistent naming</t>
         </is>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="42" t="inlineStr">
+      <c r="A14" s="43" t="inlineStr">
         <is>
           <t>Style Code / Colour Code / Option (cols B-D)</t>
         </is>
       </c>
-      <c r="B14" s="42" t="inlineStr">
+      <c r="B14" s="43" t="inlineStr">
         <is>
           <t>Not filled in for any row except the example (row 2). Also, row 2's own Option (900196AUBE) does not actually match its own Style Code (900000) or Sku - the example itself contains an inconsistency.</t>
         </is>
       </c>
-      <c r="C14" s="42" t="inlineStr">
+      <c r="C14" s="43" t="inlineStr">
         <is>
           <t>Derived Style Code and Colour Code directly from each Sku (first 6 digits / the 4 letters between 'ZZ' and the trailing '0000'), and built Option as Style Code + Colour Code consistently for every row.</t>
         </is>
       </c>
-      <c r="D14" s="42" t="inlineStr">
+      <c r="D14" s="43" t="inlineStr">
         <is>
           <t>Missing data + example inconsistency</t>
         </is>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="42" t="inlineStr">
+      <c r="A15" s="43" t="inlineStr">
         <is>
           <t>Category / Material / Style (cols E-G)</t>
         </is>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B15" s="43" t="inlineStr">
         <is>
           <t>Not filled in for any row.</t>
         </is>
       </c>
-      <c r="C15" s="42" t="inlineStr">
+      <c r="C15" s="43" t="inlineStr">
         <is>
           <t>Derived from the 6-digit style-code prefix of the Sku (e.g. 900236 = Fingerless Gloves), cross-checked against the product names on the ReBorn reference tab.</t>
         </is>
       </c>
-      <c r="D15" s="42" t="inlineStr">
+      <c r="D15" s="43" t="inlineStr">
         <is>
           <t>Missing data</t>
         </is>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="42" t="inlineStr">
+      <c r="A16" s="43" t="inlineStr">
         <is>
           <t>Colour (col I)</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B16" s="43" t="inlineStr">
         <is>
           <t>Not filled in for any row.</t>
         </is>
       </c>
-      <c r="C16" s="42" t="inlineStr">
+      <c r="C16" s="43" t="inlineStr">
         <is>
           <t>Extracted from the middle segment of each Description (text between the two commas).</t>
         </is>
       </c>
-      <c r="D16" s="42" t="inlineStr">
+      <c r="D16" s="43" t="inlineStr">
         <is>
           <t>Missing data</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="42" t="inlineStr">
+      <c r="A17" s="43" t="inlineStr">
         <is>
           <t>Size (col J)</t>
         </is>
       </c>
-      <c r="B17" s="42" t="inlineStr">
+      <c r="B17" s="43" t="inlineStr">
         <is>
           <t>Not filled in for any row.</t>
         </is>
       </c>
-      <c r="C17" s="42" t="inlineStr">
+      <c r="C17" s="43" t="inlineStr">
         <is>
           <t>Set to 'One Size' for every row - every product in this list is O/S (one size).</t>
         </is>
       </c>
-      <c r="D17" s="42" t="inlineStr">
+      <c r="D17" s="43" t="inlineStr">
         <is>
           <t>Missing data</t>
         </is>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="42" t="inlineStr">
+      <c r="A18" s="43" t="inlineStr">
         <is>
           <t>Landed Cost Price / RRP / Vat (cols M-O)</t>
         </is>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B18" s="43" t="inlineStr">
         <is>
           <t>Not filled in for any row.</t>
         </is>
       </c>
-      <c r="C18" s="42" t="inlineStr">
+      <c r="C18" s="43" t="inlineStr">
         <is>
           <t>Looked up from the ReBorn reference tab by product category and applied to every row in that category.</t>
         </is>
       </c>
-      <c r="D18" s="42" t="inlineStr">
+      <c r="D18" s="43" t="inlineStr">
         <is>
           <t>Missing data</t>
         </is>
       </c>
     </row>
     <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="42" t="inlineStr">
+      <c r="A19" s="43" t="inlineStr">
         <is>
           <t>Net RRP / Margin (cols P-Q)</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B19" s="43" t="inlineStr">
         <is>
           <t>Not filled in for any row.</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C19" s="43" t="inlineStr">
         <is>
           <t>Copied the same formulas used in the row 2 example (Net RRP = RRP/Vat, Margin = (Net RRP - Cost)/Net RRP) down every row where RRP is known.</t>
         </is>
       </c>
-      <c r="D19" s="42" t="inlineStr">
+      <c r="D19" s="43" t="inlineStr">
         <is>
           <t>Missing data</t>
         </is>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="42" t="inlineStr">
+      <c r="A20" s="43" t="inlineStr">
         <is>
           <t>2 Pack Gloves pricing (style 900235)</t>
         </is>
       </c>
-      <c r="B20" s="42" t="inlineStr">
+      <c r="B20" s="43" t="inlineStr">
         <is>
           <t>This product line (several rows) has no matching entry anywhere on the ReBorn reference tab, so Cost Price, RRP and Vat are all unknown.</t>
         </is>
       </c>
-      <c r="C20" s="42" t="inlineStr">
+      <c r="C20" s="43" t="inlineStr">
         <is>
           <t>Left marked 'TBC' (highlighted) in Cost Price, RRP, Vat, Net RRP and Margin. Recommend checking with the buying/finance team for the correct figures.</t>
         </is>
       </c>
-      <c r="D20" s="42" t="inlineStr">
+      <c r="D20" s="43" t="inlineStr">
         <is>
           <t>Further investigation needed</t>
         </is>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="42" t="inlineStr">
+      <c r="A21" s="43" t="inlineStr">
         <is>
           <t>Snood &amp; Glove Set / Beanie &amp; Glove Set RRP</t>
         </is>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B21" s="43" t="inlineStr">
         <is>
           <t>The ReBorn reference tab lists the RRP for these two lines as '?' - i.e. genuinely not yet decided/confirmed, not a data entry gap.</t>
         </is>
       </c>
-      <c r="C21" s="42" t="inlineStr">
+      <c r="C21" s="43" t="inlineStr">
         <is>
           <t>Cost Price and Vat filled in from the reference tab; RRP, Net RRP and Margin left as 'TBC' (highlighted) since inventing a number would be misleading. Recommend confirming with pricing/marketing.</t>
         </is>
       </c>
-      <c r="D21" s="42" t="inlineStr">
+      <c r="D21" s="43" t="inlineStr">
         <is>
           <t>Further investigation needed</t>
         </is>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="42" t="inlineStr">
+      <c r="A22" s="43" t="inlineStr">
         <is>
           <t>Range (col H)</t>
         </is>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B22" s="43" t="inlineStr">
         <is>
           <t>The row 2 example shows a Range of 'Core', but no other row, sheet, or column in the source data indicates what Range/Collection any product belongs to.</t>
         </is>
       </c>
-      <c r="C22" s="42" t="inlineStr">
+      <c r="C22" s="43" t="inlineStr">
         <is>
           <t>Left as 'TBC' (highlighted) for every row rather than guessing. Recommend checking with merchandising for the correct Range per style.</t>
         </is>
       </c>
-      <c r="D22" s="42" t="inlineStr">
+      <c r="D22" s="43" t="inlineStr">
         <is>
           <t>Further investigation needed</t>
         </is>

</xml_diff>